<commit_message>
moved loading out of sight
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{127086A6-DFCE-EC42-BEBA-E6222BE726E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9440D2-5C4A-2043-948C-627C5A6DA88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="34740" yWindow="4480" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -937,18 +937,44 @@
         <v>2061</v>
       </c>
       <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="6"/>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
-      <c r="S2" s="6"/>
-      <c r="T2" s="6"/>
+      <c r="I2" s="6">
+        <v>6801</v>
+      </c>
+      <c r="J2" s="6">
+        <v>1.56</v>
+      </c>
+      <c r="K2" s="6">
+        <v>1.43</v>
+      </c>
+      <c r="L2" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="M2" s="6">
+        <v>4.21</v>
+      </c>
+      <c r="N2" s="6">
+        <v>7.3289156000000002</v>
+      </c>
+      <c r="O2" s="6">
+        <v>-76.304032000000007</v>
+      </c>
+      <c r="P2" s="6">
+        <v>196.852</v>
+      </c>
+      <c r="Q2" s="6">
+        <v>9.5950000000000006</v>
+      </c>
+      <c r="R2" s="6">
+        <v>9.5202500000000008</v>
+      </c>
+      <c r="S2" s="6">
+        <f t="shared" ref="S2:S33" si="0">(0.000000000000000138*G2/(1.673534E-24*1.3*0.000000066726*F2*1.8986E+30/(E2*7149200000)^2))/100000</f>
+        <v>934.76971602454307</v>
+      </c>
+      <c r="T2" s="6">
+        <f t="shared" ref="T2:T33" si="1">IF(I2&gt;6800,-7,-5)</f>
+        <v>-7</v>
+      </c>
       <c r="U2" s="7" t="s">
         <v>138</v>
       </c>
@@ -1012,11 +1038,11 @@
         <v>7.5767499999999997</v>
       </c>
       <c r="S3" s="6">
-        <f t="shared" ref="S2:S33" si="0">(0.000000000000000138*G3/(1.673534E-24*1.3*0.000000066726*F3*1.8986E+30/(E3*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1286.8653667451285</v>
       </c>
       <c r="T3" s="6">
-        <f t="shared" ref="T2:T33" si="1">IF(I3&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
       <c r="U3" s="7" t="s">

</xml_diff>

<commit_message>
introducted gaia only required keys. so that gaia lookup only occurs for gaia keys
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA9440D2-5C4A-2043-948C-627C5A6DA88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02884B69-2385-A341-98C4-5D1D351D5428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="34740" yWindow="4480" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added some backgroudn info
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A350165-11CD-384A-97C3-9E8028631666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8F862D4-3F96-2D46-9781-6AA4098864CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="14820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17740" yWindow="1780" windowWidth="33600" windowHeight="25500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="141">
   <si>
     <t>#pl_name</t>
   </si>
@@ -456,6 +456,9 @@
   </si>
   <si>
     <t>WASP-12 b</t>
+  </si>
+  <si>
+    <t>eps boo b</t>
   </si>
 </sst>
 </file>
@@ -831,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH80"/>
+  <dimension ref="A1:BH81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
@@ -986,11 +989,11 @@
         <v>10.178599999999999</v>
       </c>
       <c r="S2">
-        <f>(0.000000000000000138*G2/(1.673534E-24*1.3*0.000000066726*F2*1.8986E+30/(E2*7149200000)^2))/100000</f>
+        <f t="shared" ref="S2:S33" si="0">(0.000000000000000138*G2/(1.673534E-24*1.3*0.000000066726*F2*1.8986E+30/(E2*7149200000)^2))/100000</f>
         <v>1121.1126749906216</v>
       </c>
       <c r="T2">
-        <f>IF(I2&gt;6800,-7,-5)</f>
+        <f t="shared" ref="T2:T33" si="1">IF(I2&gt;6800,-7,-5)</f>
         <v>-5</v>
       </c>
       <c r="BE2" s="3"/>
@@ -1053,11 +1056,11 @@
         <v>9.8728300000000004</v>
       </c>
       <c r="S3">
-        <f>(0.000000000000000138*G3/(1.673534E-24*1.3*0.000000066726*F3*1.8986E+30/(E3*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>243.60813720463176</v>
       </c>
       <c r="T3">
-        <f>IF(I3&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="BE3" s="3"/>
@@ -1120,11 +1123,11 @@
         <v>8.5984200000000008</v>
       </c>
       <c r="S4">
-        <f>(0.000000000000000138*G4/(1.673534E-24*1.3*0.000000066726*F4*1.8986E+30/(E4*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>39.515068300859213</v>
       </c>
       <c r="T4">
-        <f>IF(I4&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="BE4" s="3"/>
@@ -1187,11 +1190,11 @@
         <v>9.5193600000000007</v>
       </c>
       <c r="S5">
-        <f>(0.000000000000000138*G5/(1.673534E-24*1.3*0.000000066726*F5*1.8986E+30/(E5*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>200.46131426194896</v>
       </c>
       <c r="T5">
-        <f>IF(I5&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="BE5" s="3"/>
@@ -1251,11 +1254,11 @@
         <v>9.5635499999999993</v>
       </c>
       <c r="S6">
-        <f>(0.000000000000000138*G6/(1.673534E-24*1.3*0.000000066726*F6*1.8986E+30/(E6*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>2101.5864855136347</v>
       </c>
       <c r="T6">
-        <f>IF(I6&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="BE6" s="3"/>
@@ -1315,11 +1318,11 @@
         <v>9.77332</v>
       </c>
       <c r="S7">
-        <f>(0.000000000000000138*G7/(1.673534E-24*1.3*0.000000066726*F7*1.8986E+30/(E7*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>387.53401759458865</v>
       </c>
       <c r="T7">
-        <f>IF(I7&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
       <c r="V7" s="2"/>
@@ -1379,11 +1382,11 @@
         <v>9.4517399999999991</v>
       </c>
       <c r="S8">
-        <f>(0.000000000000000138*G8/(1.673534E-24*1.3*0.000000066726*F8*1.8986E+30/(E8*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>338.15838787809196</v>
       </c>
       <c r="T8">
-        <f>IF(I8&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
       <c r="V8" s="2"/>
@@ -1446,11 +1449,11 @@
         <v>7.89255</v>
       </c>
       <c r="S9">
-        <f>(0.000000000000000138*G9/(1.673534E-24*1.3*0.000000066726*F9*1.8986E+30/(E9*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>211.51519610586323</v>
       </c>
       <c r="T9">
-        <f>IF(I9&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1510,11 +1513,11 @@
         <v>7.5933599999999997</v>
       </c>
       <c r="S10">
-        <f>(0.000000000000000138*G10/(1.673534E-24*1.3*0.000000066726*F10*1.8986E+30/(E10*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>797.33090232058362</v>
       </c>
       <c r="T10">
-        <f>IF(I10&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1574,11 +1577,11 @@
         <v>8.0141600000000004</v>
       </c>
       <c r="S11">
-        <f>(0.000000000000000138*G11/(1.673534E-24*1.3*0.000000066726*F11*1.8986E+30/(E11*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>599.63628364223177</v>
       </c>
       <c r="T11">
-        <f>IF(I11&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="V11" s="2"/>
@@ -1641,11 +1644,11 @@
         <v>8.7641200000000001</v>
       </c>
       <c r="S12">
-        <f>(0.000000000000000138*G12/(1.673534E-24*1.3*0.000000066726*F12*1.8986E+30/(E12*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>597.79498778467087</v>
       </c>
       <c r="T12">
-        <f>IF(I12&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1705,11 +1708,11 @@
         <v>7.41432</v>
       </c>
       <c r="S13">
-        <f>(0.000000000000000138*G13/(1.673534E-24*1.3*0.000000066726*F13*1.8986E+30/(E13*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>349.61677638948368</v>
       </c>
       <c r="T13">
-        <f>IF(I13&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1766,11 +1769,11 @@
         <v>8.2268799999999995</v>
       </c>
       <c r="S14">
-        <f>(0.000000000000000138*G14/(1.673534E-24*1.3*0.000000066726*F14*1.8986E+30/(E14*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1280.5918535006856</v>
       </c>
       <c r="T14">
-        <f>IF(I14&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="V14" s="2"/>
@@ -1833,11 +1836,11 @@
         <v>7.5086599999999999</v>
       </c>
       <c r="S15">
-        <f>(0.000000000000000138*G15/(1.673534E-24*1.3*0.000000066726*F15*1.8986E+30/(E15*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>988.21070019970352</v>
       </c>
       <c r="T15">
-        <f>IF(I15&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1897,11 +1900,11 @@
         <v>9.6495599999999992</v>
       </c>
       <c r="S16">
-        <f>(0.000000000000000138*G16/(1.673534E-24*1.3*0.000000066726*F16*1.8986E+30/(E16*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>956.09264119622901</v>
       </c>
       <c r="T16">
-        <f>IF(I16&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="V16" s="2"/>
@@ -1964,11 +1967,11 @@
         <v>7.9077599999999997</v>
       </c>
       <c r="S17">
-        <f>(0.000000000000000138*G17/(1.673534E-24*1.3*0.000000066726*F17*1.8986E+30/(E17*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>742.8583931109747</v>
       </c>
       <c r="T17">
-        <f>IF(I17&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2026,11 +2029,11 @@
         <v>9.5202500000000008</v>
       </c>
       <c r="S18" s="6">
-        <f>(0.000000000000000138*G18/(1.673534E-24*1.3*0.000000066726*F18*1.8986E+30/(E18*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>934.76971602454307</v>
       </c>
       <c r="T18" s="6">
-        <f>IF(I18&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
       <c r="U18" s="7" t="s">
@@ -2093,11 +2096,11 @@
         <v>8.4183900000000005</v>
       </c>
       <c r="S19">
-        <f>(0.000000000000000138*G19/(1.673534E-24*1.3*0.000000066726*F19*1.8986E+30/(E19*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>574.11765847468712</v>
       </c>
       <c r="T19">
-        <f>IF(I19&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2157,11 +2160,11 @@
         <v>7.8097899999999996</v>
       </c>
       <c r="S20">
-        <f>(0.000000000000000138*G20/(1.673534E-24*1.3*0.000000066726*F20*1.8986E+30/(E20*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>668.81110409377118</v>
       </c>
       <c r="T20">
-        <f>IF(I20&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2221,11 +2224,11 @@
         <v>9.2170199999999998</v>
       </c>
       <c r="S21">
-        <f>(0.000000000000000138*G21/(1.673534E-24*1.3*0.000000066726*F21*1.8986E+30/(E21*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1103.5971886171305</v>
       </c>
       <c r="T21">
-        <f>IF(I21&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2282,11 +2285,11 @@
         <v>9.7262599999999999</v>
       </c>
       <c r="S22">
-        <f>(0.000000000000000138*G22/(1.673534E-24*1.3*0.000000066726*F22*1.8986E+30/(E22*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>662.28004924519439</v>
       </c>
       <c r="T22">
-        <f>IF(I22&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2346,11 +2349,11 @@
         <v>7.8311200000000003</v>
       </c>
       <c r="S23">
-        <f>(0.000000000000000138*G23/(1.673534E-24*1.3*0.000000066726*F23*1.8986E+30/(E23*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>3894.9775251994533</v>
       </c>
       <c r="T23">
-        <f>IF(I23&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2410,11 +2413,11 @@
         <v>9.2088699999999992</v>
       </c>
       <c r="S24">
-        <f>(0.000000000000000138*G24/(1.673534E-24*1.3*0.000000066726*F24*1.8986E+30/(E24*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>948.15286253702118</v>
       </c>
       <c r="T24">
-        <f>IF(I24&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -2474,11 +2477,11 @@
         <v>9.8633100000000002</v>
       </c>
       <c r="S25">
-        <f>(0.000000000000000138*G25/(1.673534E-24*1.3*0.000000066726*F25*1.8986E+30/(E25*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>443.85469120292152</v>
       </c>
       <c r="T25">
-        <f>IF(I25&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -2538,11 +2541,11 @@
         <v>8.5839300000000005</v>
       </c>
       <c r="S26">
-        <f>(0.000000000000000138*G26/(1.673534E-24*1.3*0.000000066726*F26*1.8986E+30/(E26*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>570.64953846380126</v>
       </c>
       <c r="T26">
-        <f>IF(I26&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2602,11 +2605,11 @@
         <v>7.5749199999999997</v>
       </c>
       <c r="S27">
-        <f>(0.000000000000000138*G27/(1.673534E-24*1.3*0.000000066726*F27*1.8986E+30/(E27*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>518.80488815900412</v>
       </c>
       <c r="T27">
-        <f>IF(I27&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -2666,11 +2669,11 @@
         <v>8.23752</v>
       </c>
       <c r="S28">
-        <f>(0.000000000000000138*G28/(1.673534E-24*1.3*0.000000066726*F28*1.8986E+30/(E28*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>99.730517672190274</v>
       </c>
       <c r="T28">
-        <f>IF(I28&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2727,11 +2730,11 @@
         <v>9.7632399999999997</v>
       </c>
       <c r="S29">
-        <f>(0.000000000000000138*G29/(1.673534E-24*1.3*0.000000066726*F29*1.8986E+30/(E29*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>582.97620763372299</v>
       </c>
       <c r="T29">
-        <f>IF(I29&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2791,11 +2794,11 @@
         <v>9.95702</v>
       </c>
       <c r="S30">
-        <f>(0.000000000000000138*G30/(1.673534E-24*1.3*0.000000066726*F30*1.8986E+30/(E30*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1492.9814393090719</v>
       </c>
       <c r="T30">
-        <f>IF(I30&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2855,11 +2858,11 @@
         <v>8.4517299999999995</v>
       </c>
       <c r="S31">
-        <f>(0.000000000000000138*G31/(1.673534E-24*1.3*0.000000066726*F31*1.8986E+30/(E31*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>965.25628287035329</v>
       </c>
       <c r="T31">
-        <f>IF(I31&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2919,11 +2922,11 @@
         <v>7.5767499999999997</v>
       </c>
       <c r="S32" s="6">
-        <f>(0.000000000000000138*G32/(1.673534E-24*1.3*0.000000066726*F32*1.8986E+30/(E32*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1286.8653667451285</v>
       </c>
       <c r="T32" s="6">
-        <f>IF(I32&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
       <c r="U32" s="7" t="s">
@@ -2983,11 +2986,11 @@
         <v>10.367800000000001</v>
       </c>
       <c r="S33">
-        <f>(0.000000000000000138*G33/(1.673534E-24*1.3*0.000000066726*F33*1.8986E+30/(E33*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>160.76196513632402</v>
       </c>
       <c r="T33">
-        <f>IF(I33&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -3047,11 +3050,11 @@
         <v>9.6000599999999991</v>
       </c>
       <c r="S34">
-        <f>(0.000000000000000138*G34/(1.673534E-24*1.3*0.000000066726*F34*1.8986E+30/(E34*7149200000)^2))/100000</f>
+        <f t="shared" ref="S34:S59" si="2">(0.000000000000000138*G34/(1.673534E-24*1.3*0.000000066726*F34*1.8986E+30/(E34*7149200000)^2))/100000</f>
         <v>972.96006983022733</v>
       </c>
       <c r="T34">
-        <f>IF(I34&gt;6800,-7,-5)</f>
+        <f t="shared" ref="T34:T65" si="3">IF(I34&gt;6800,-7,-5)</f>
         <v>-5</v>
       </c>
     </row>
@@ -3111,11 +3114,11 @@
         <v>8.2424300000000006</v>
       </c>
       <c r="S35">
-        <f>(0.000000000000000138*G35/(1.673534E-24*1.3*0.000000066726*F35*1.8986E+30/(E35*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>457.63140850776114</v>
       </c>
       <c r="T35">
-        <f>IF(I35&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3175,11 +3178,11 @@
         <v>8.1740100000000009</v>
       </c>
       <c r="S36">
-        <f>(0.000000000000000138*G36/(1.673534E-24*1.3*0.000000066726*F36*1.8986E+30/(E36*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>789.006338593706</v>
       </c>
       <c r="T36">
-        <f>IF(I36&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3239,11 +3242,11 @@
         <v>9.4290710000000004</v>
       </c>
       <c r="S37" s="6">
-        <f>(0.000000000000000138*G37/(1.673534E-24*1.3*0.000000066726*F37*1.8986E+30/(E37*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>56.120615203365361</v>
       </c>
       <c r="T37" s="6">
-        <f>IF(I37&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
       <c r="U37" s="7" t="s">
@@ -3306,11 +3309,11 @@
         <v>9.4135299999999997</v>
       </c>
       <c r="S38">
-        <f>(0.000000000000000138*G38/(1.673534E-24*1.3*0.000000066726*F38*1.8986E+30/(E38*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1175.9460676296278</v>
       </c>
       <c r="T38">
-        <f>IF(I38&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3367,11 +3370,11 @@
         <v>9.3678899999999992</v>
       </c>
       <c r="S39">
-        <f>(0.000000000000000138*G39/(1.673534E-24*1.3*0.000000066726*F39*1.8986E+30/(E39*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1399.2265914107247</v>
       </c>
       <c r="T39">
-        <f>IF(I39&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3428,11 +3431,11 @@
         <v>9.3503900000000009</v>
       </c>
       <c r="S40">
-        <f>(0.000000000000000138*G40/(1.673534E-24*1.3*0.000000066726*F40*1.8986E+30/(E40*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>353.31388599481477</v>
       </c>
       <c r="T40">
-        <f>IF(I40&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3492,11 +3495,11 @@
         <v>9.1879500000000007</v>
       </c>
       <c r="S41">
-        <f>(0.000000000000000138*G41/(1.673534E-24*1.3*0.000000066726*F41*1.8986E+30/(E41*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>882.20971786077962</v>
       </c>
       <c r="T41">
-        <f>IF(I41&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3556,11 +3559,11 @@
         <v>7.9756099999999996</v>
       </c>
       <c r="S42">
-        <f>(0.000000000000000138*G42/(1.673534E-24*1.3*0.000000066726*F42*1.8986E+30/(E42*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>431.57254486096394</v>
       </c>
       <c r="T42">
-        <f>IF(I42&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3620,11 +3623,11 @@
         <v>8.8952899999999993</v>
       </c>
       <c r="S43">
-        <f>(0.000000000000000138*G43/(1.673534E-24*1.3*0.000000066726*F43*1.8986E+30/(E43*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>974.78820571370204</v>
       </c>
       <c r="T43">
-        <f>IF(I43&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3684,11 +3687,11 @@
         <v>9.5843900000000009</v>
       </c>
       <c r="S44">
-        <f>(0.000000000000000138*G44/(1.673534E-24*1.3*0.000000066726*F44*1.8986E+30/(E44*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1460.8182255852041</v>
       </c>
       <c r="T44">
-        <f>IF(I44&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3745,11 +3748,11 @@
         <v>9.6598100000000002</v>
       </c>
       <c r="S45">
-        <f>(0.000000000000000138*G45/(1.673534E-24*1.3*0.000000066726*F45*1.8986E+30/(E45*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1324.5165539963698</v>
       </c>
       <c r="T45">
-        <f>IF(I45&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3806,11 +3809,11 @@
         <v>9.7596699999999998</v>
       </c>
       <c r="S46">
-        <f>(0.000000000000000138*G46/(1.673534E-24*1.3*0.000000066726*F46*1.8986E+30/(E46*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>55.915145726222889</v>
       </c>
       <c r="T46">
-        <f>IF(I46&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3867,11 +3870,11 @@
         <v>8.9365100000000002</v>
       </c>
       <c r="S47">
-        <f>(0.000000000000000138*G47/(1.673534E-24*1.3*0.000000066726*F47*1.8986E+30/(E47*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>77.040187113891676</v>
       </c>
       <c r="T47">
-        <f>IF(I47&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3928,11 +3931,11 @@
         <v>9.4724400000000006</v>
       </c>
       <c r="S48">
-        <f>(0.000000000000000138*G48/(1.673534E-24*1.3*0.000000066726*F48*1.8986E+30/(E48*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>83.670803141549356</v>
       </c>
       <c r="T48">
-        <f>IF(I48&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3989,11 +3992,11 @@
         <v>7.4165299999999998</v>
       </c>
       <c r="S49">
-        <f>(0.000000000000000138*G49/(1.673534E-24*1.3*0.000000066726*F49*1.8986E+30/(E49*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>777.64358420307099</v>
       </c>
       <c r="T49">
-        <f>IF(I49&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4053,11 +4056,11 @@
         <v>9.7777600000000007</v>
       </c>
       <c r="S50">
-        <f>(0.000000000000000138*G50/(1.673534E-24*1.3*0.000000066726*F50*1.8986E+30/(E50*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>755.33252275944176</v>
       </c>
       <c r="T50">
-        <f>IF(I50&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4114,11 +4117,11 @@
         <v>9.641</v>
       </c>
       <c r="S51">
-        <f>(0.000000000000000138*G51/(1.673534E-24*1.3*0.000000066726*F51*1.8986E+30/(E51*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>318.17832033985127</v>
       </c>
       <c r="T51">
-        <f>IF(I51&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4178,11 +4181,11 @@
         <v>9.0746900000000004</v>
       </c>
       <c r="S52">
-        <f>(0.000000000000000138*G52/(1.673534E-24*1.3*0.000000066726*F52*1.8986E+30/(E52*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>36.149567272802649</v>
       </c>
       <c r="T52">
-        <f>IF(I52&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4242,11 +4245,11 @@
         <v>9.8465900000000008</v>
       </c>
       <c r="S53">
-        <f>(0.000000000000000138*G53/(1.673534E-24*1.3*0.000000066726*F53*1.8986E+30/(E53*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>224.58825733889913</v>
       </c>
       <c r="T53">
-        <f>IF(I53&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4303,11 +4306,11 @@
         <v>9.6080000000000005</v>
       </c>
       <c r="S54">
-        <f>(0.000000000000000138*G54/(1.673534E-24*1.3*0.000000066726*F54*1.8986E+30/(E54*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1039.84328949877</v>
       </c>
       <c r="T54">
-        <f>IF(I54&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4367,11 +4370,11 @@
         <v>9.9823299999999993</v>
       </c>
       <c r="S55">
-        <f>(0.000000000000000138*G55/(1.673534E-24*1.3*0.000000066726*F55*1.8986E+30/(E55*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1107.9861243219782</v>
       </c>
       <c r="T55">
-        <f>IF(I55&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4428,11 +4431,11 @@
         <v>9.7295700000000007</v>
       </c>
       <c r="S56">
-        <f>(0.000000000000000138*G56/(1.673534E-24*1.3*0.000000066726*F56*1.8986E+30/(E56*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>487.59044264912109</v>
       </c>
       <c r="T56">
-        <f>IF(I56&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4492,11 +4495,11 @@
         <v>8.8910300000000007</v>
       </c>
       <c r="S57">
-        <f>(0.000000000000000138*G57/(1.673534E-24*1.3*0.000000066726*F57*1.8986E+30/(E57*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>795.95548671567838</v>
       </c>
       <c r="T57">
-        <f>IF(I57&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4556,11 +4559,11 @@
         <v>9.6608199999999993</v>
       </c>
       <c r="S58">
-        <f>(0.000000000000000138*G58/(1.673534E-24*1.3*0.000000066726*F58*1.8986E+30/(E58*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>355.42536038318485</v>
       </c>
       <c r="T58">
-        <f>IF(I58&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4620,11 +4623,11 @@
         <v>8.9943600000000004</v>
       </c>
       <c r="S59">
-        <f>(0.000000000000000138*G59/(1.673534E-24*1.3*0.000000066726*F59*1.8986E+30/(E59*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>267.77715667890726</v>
       </c>
       <c r="T59">
-        <f>IF(I59&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4654,7 +4657,7 @@
         <v>11.4986</v>
       </c>
       <c r="T60">
-        <f>IF(I60&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4714,11 +4717,11 @@
         <v>9.8670799999999996</v>
       </c>
       <c r="S61">
-        <f>(0.000000000000000138*G61/(1.673534E-24*1.3*0.000000066726*F61*1.8986E+30/(E61*7149200000)^2))/100000</f>
+        <f t="shared" ref="S61:S80" si="4">(0.000000000000000138*G61/(1.673534E-24*1.3*0.000000066726*F61*1.8986E+30/(E61*7149200000)^2))/100000</f>
         <v>2057.1154637812851</v>
       </c>
       <c r="T61">
-        <f>IF(I61&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4778,11 +4781,11 @@
         <v>9.8192900000000005</v>
       </c>
       <c r="S62">
-        <f>(0.000000000000000138*G62/(1.673534E-24*1.3*0.000000066726*F62*1.8986E+30/(E62*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>621.55661806820979</v>
       </c>
       <c r="T62">
-        <f>IF(I62&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4839,11 +4842,11 @@
         <v>9.6464700000000008</v>
       </c>
       <c r="S63">
-        <f>(0.000000000000000138*G63/(1.673534E-24*1.3*0.000000066726*F63*1.8986E+30/(E63*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>103.20465157174387</v>
       </c>
       <c r="T63">
-        <f>IF(I63&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4903,11 +4906,11 @@
         <v>9.2569999999999997</v>
       </c>
       <c r="S64">
-        <f>(0.000000000000000138*G64/(1.673534E-24*1.3*0.000000066726*F64*1.8986E+30/(E64*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>1277.1766379712274</v>
       </c>
       <c r="T64">
-        <f>IF(I64&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4967,11 +4970,11 @@
         <v>9.9122599999999998</v>
       </c>
       <c r="S65">
-        <f>(0.000000000000000138*G65/(1.673534E-24*1.3*0.000000066726*F65*1.8986E+30/(E65*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>1247.4798366438731</v>
       </c>
       <c r="T65">
-        <f>IF(I65&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -5031,11 +5034,11 @@
         <v>9.1661699999999993</v>
       </c>
       <c r="S66">
-        <f>(0.000000000000000138*G66/(1.673534E-24*1.3*0.000000066726*F66*1.8986E+30/(E66*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>93.704022194109143</v>
       </c>
       <c r="T66">
-        <f>IF(I66&gt;6800,-7,-5)</f>
+        <f t="shared" ref="T66:T80" si="5">IF(I66&gt;6800,-7,-5)</f>
         <v>-5</v>
       </c>
     </row>
@@ -5093,11 +5096,11 @@
         <v>6.5536899999999996</v>
       </c>
       <c r="S67" s="8">
-        <f>(0.000000000000000138*G67/(1.673534E-24*1.3*0.000000066726*F67*1.8986E+30/(E67*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>1130.2166328238993</v>
       </c>
       <c r="T67" s="6">
-        <f>IF(I67&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-7</v>
       </c>
       <c r="U67" s="7" t="s">
@@ -5160,11 +5163,11 @@
         <v>8.0700400000000005</v>
       </c>
       <c r="S68">
-        <f>(0.000000000000000138*G68/(1.673534E-24*1.3*0.000000066726*F68*1.8986E+30/(E68*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>863.09804630713359</v>
       </c>
       <c r="T68">
-        <f>IF(I68&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-7</v>
       </c>
     </row>
@@ -5224,11 +5227,11 @@
         <v>9.20974</v>
       </c>
       <c r="S69">
-        <f>(0.000000000000000138*G69/(1.673534E-24*1.3*0.000000066726*F69*1.8986E+30/(E69*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>140.68549179703928</v>
       </c>
       <c r="T69">
-        <f>IF(I69&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5288,11 +5291,11 @@
         <v>9.4846599999999999</v>
       </c>
       <c r="S70" s="6">
-        <f>(0.000000000000000138*G70/(1.673534E-24*1.3*0.000000066726*F70*1.8986E+30/(E70*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>955.72600175951948</v>
       </c>
       <c r="T70" s="6">
-        <f>IF(I70&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
       <c r="U70" s="7" t="s">
@@ -5352,11 +5355,11 @@
         <v>9.3767099999999992</v>
       </c>
       <c r="S71">
-        <f>(0.000000000000000138*G71/(1.673534E-24*1.3*0.000000066726*F71*1.8986E+30/(E71*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>701.18164217622461</v>
       </c>
       <c r="T71">
-        <f>IF(I71&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5416,11 +5419,11 @@
         <v>9.5723000000000003</v>
       </c>
       <c r="S72">
-        <f>(0.000000000000000138*G72/(1.673534E-24*1.3*0.000000066726*F72*1.8986E+30/(E72*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>1226.0598654781754</v>
       </c>
       <c r="T72">
-        <f>IF(I72&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5480,11 +5483,11 @@
         <v>9.3950700000000005</v>
       </c>
       <c r="S73">
-        <f>(0.000000000000000138*G73/(1.673534E-24*1.3*0.000000066726*F73*1.8986E+30/(E73*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>2192.2225820487197</v>
       </c>
       <c r="T73">
-        <f>IF(I73&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5544,11 +5547,11 @@
         <v>9.9720200000000006</v>
       </c>
       <c r="S74">
-        <f>(0.000000000000000138*G74/(1.673534E-24*1.3*0.000000066726*F74*1.8986E+30/(E74*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>1209.5375438309629</v>
       </c>
       <c r="T74">
-        <f>IF(I74&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5608,11 +5611,11 @@
         <v>9.6124899999999993</v>
       </c>
       <c r="S75">
-        <f>(0.000000000000000138*G75/(1.673534E-24*1.3*0.000000066726*F75*1.8986E+30/(E75*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>136.24063220140397</v>
       </c>
       <c r="T75">
-        <f>IF(I75&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5672,11 +5675,11 @@
         <v>9.8979599999999994</v>
       </c>
       <c r="S76">
-        <f>(0.000000000000000138*G76/(1.673534E-24*1.3*0.000000066726*F76*1.8986E+30/(E76*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>1257.117296864338</v>
       </c>
       <c r="T76">
-        <f>IF(I76&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5736,11 +5739,11 @@
         <v>10.028499999999999</v>
       </c>
       <c r="S77">
-        <f>(0.000000000000000138*G77/(1.673534E-24*1.3*0.000000066726*F77*1.8986E+30/(E77*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>2049.4439875099679</v>
       </c>
       <c r="T77">
-        <f>IF(I77&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5800,11 +5803,11 @@
         <v>9.9369700000000005</v>
       </c>
       <c r="S78">
-        <f>(0.000000000000000138*G78/(1.673534E-24*1.3*0.000000066726*F78*1.8986E+30/(E78*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>422.11900227636102</v>
       </c>
       <c r="T78">
-        <f>IF(I78&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5864,11 +5867,11 @@
         <v>9.3251000000000008</v>
       </c>
       <c r="S79">
-        <f>(0.000000000000000138*G79/(1.673534E-24*1.3*0.000000066726*F79*1.8986E+30/(E79*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>162.15983922320817</v>
       </c>
       <c r="T79">
-        <f>IF(I79&gt;6800,-7,-5)</f>
+        <f t="shared" si="5"/>
         <v>-5</v>
       </c>
     </row>
@@ -5928,12 +5931,17 @@
         <v>9.7388899999999996</v>
       </c>
       <c r="S80">
-        <f>(0.000000000000000138*G80/(1.673534E-24*1.3*0.000000066726*F80*1.8986E+30/(E80*7149200000)^2))/100000</f>
+        <f t="shared" si="4"/>
         <v>120.66830436099001</v>
       </c>
       <c r="T80">
-        <f>IF(I80&gt;6800,-7,-5)</f>
-        <v>-5</v>
+        <f t="shared" si="5"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" s="4" t="s">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added nuv, vis, nir specific config until convolution
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/waltzerclone/WALTzER-simulator/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2DC096E-5C4E-9D4F-9092-4AD1AC0C6EB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D4D5BB-BFFC-0C4C-988C-A73FCF734FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="2200" windowWidth="33600" windowHeight="25500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22040" yWindow="820" windowWidth="33600" windowHeight="25500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="145">
   <si>
     <t>#pl_name</t>
   </si>
@@ -468,6 +468,9 @@
   </si>
   <si>
     <t>TrES-4 b</t>
+  </si>
+  <si>
+    <t>B9.5-A0</t>
   </si>
 </sst>
 </file>
@@ -500,7 +503,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,6 +532,12 @@
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor theme="5" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
   </fills>
@@ -587,7 +596,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -621,26 +630,23 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1021,25 +1027,21 @@
       <c r="A2" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="H2" s="11"/>
-      <c r="I2" s="17">
+      <c r="I2" s="16">
         <v>4907.77490234375</v>
       </c>
-      <c r="J2" s="17"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17">
+      <c r="J2" s="16"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16">
         <v>221.24648617076679</v>
       </c>
-      <c r="O2" s="17">
+      <c r="O2" s="16">
         <v>27.074315757773469</v>
       </c>
-      <c r="P2" s="11"/>
-      <c r="Q2" s="17">
+      <c r="Q2" s="16">
         <v>2.1833524703979492</v>
       </c>
-      <c r="R2" s="17">
+      <c r="R2" s="16">
         <v>2.1833524703979492</v>
       </c>
       <c r="BE2" s="3"/>
@@ -1315,35 +1317,32 @@
       <c r="BH6" s="3"/>
     </row>
     <row r="7" spans="1:60" x14ac:dyDescent="0.2">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="17">
+      <c r="B7" s="14"/>
+      <c r="I7" s="16">
         <v>6245.11328125</v>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="16">
         <v>1.208241820335388</v>
       </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="17">
+      <c r="M7" s="16">
         <v>4.2744002342224121</v>
       </c>
-      <c r="N7" s="17">
+      <c r="N7" s="16">
         <v>31.04275939878713</v>
       </c>
-      <c r="O7" s="17">
+      <c r="O7" s="16">
         <v>46.687851647860192</v>
       </c>
-      <c r="P7" s="11">
+      <c r="P7">
         <v>283.38339999999999</v>
       </c>
-      <c r="Q7" s="17">
+      <c r="Q7" s="16">
         <v>11.12930202484131</v>
       </c>
-      <c r="R7" s="17">
+      <c r="R7" s="16">
         <v>11.12930202484131</v>
       </c>
       <c r="V7" s="2"/>
@@ -1476,30 +1475,26 @@
       </c>
     </row>
     <row r="10" spans="1:60" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="17">
+      <c r="I10" s="16">
         <v>6424.27685546875</v>
       </c>
-      <c r="J10" s="17">
+      <c r="J10" s="16">
         <v>2.0702402591705318</v>
       </c>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17">
+      <c r="M10" s="16"/>
+      <c r="N10" s="16">
         <v>292.24718620018581</v>
       </c>
-      <c r="O10" s="17">
+      <c r="O10" s="16">
         <v>47.969544064101818</v>
       </c>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="17">
+      <c r="Q10" s="16">
         <v>10.36768245697021</v>
       </c>
-      <c r="R10" s="17">
+      <c r="R10" s="16">
         <v>10.36768245697021</v>
       </c>
     </row>
@@ -1556,11 +1551,11 @@
         <v>9.4517399999999991</v>
       </c>
       <c r="S11">
-        <f>(0.000000000000000138*G11/(1.673534E-24*1.3*0.000000066726*F11*1.8986E+30/(E11*7149200000)^2))/100000</f>
+        <f t="shared" ref="S11:S35" si="0">(0.000000000000000138*G11/(1.673534E-24*1.3*0.000000066726*F11*1.8986E+30/(E11*7149200000)^2))/100000</f>
         <v>338.15838787809196</v>
       </c>
       <c r="T11">
-        <f>IF(I11&gt;6800,-7,-5)</f>
+        <f t="shared" ref="T11:T34" si="1">IF(I11&gt;6800,-7,-5)</f>
         <v>-7</v>
       </c>
       <c r="V11" s="2"/>
@@ -1623,11 +1618,11 @@
         <v>7.89255</v>
       </c>
       <c r="S12">
-        <f>(0.000000000000000138*G12/(1.673534E-24*1.3*0.000000066726*F12*1.8986E+30/(E12*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>211.51519610586323</v>
       </c>
       <c r="T12">
-        <f>IF(I12&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1687,11 +1682,11 @@
         <v>7.5933599999999997</v>
       </c>
       <c r="S13">
-        <f>(0.000000000000000138*G13/(1.673534E-24*1.3*0.000000066726*F13*1.8986E+30/(E13*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>797.33090232058362</v>
       </c>
       <c r="T13">
-        <f>IF(I13&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1751,11 +1746,11 @@
         <v>8.0141600000000004</v>
       </c>
       <c r="S14">
-        <f>(0.000000000000000138*G14/(1.673534E-24*1.3*0.000000066726*F14*1.8986E+30/(E14*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>599.63628364223177</v>
       </c>
       <c r="T14">
-        <f>IF(I14&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="V14" s="2"/>
@@ -1818,11 +1813,11 @@
         <v>8.7641200000000001</v>
       </c>
       <c r="S15">
-        <f>(0.000000000000000138*G15/(1.673534E-24*1.3*0.000000066726*F15*1.8986E+30/(E15*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>597.79498778467087</v>
       </c>
       <c r="T15">
-        <f>IF(I15&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -1882,11 +1877,11 @@
         <v>7.41432</v>
       </c>
       <c r="S16">
-        <f>(0.000000000000000138*G16/(1.673534E-24*1.3*0.000000066726*F16*1.8986E+30/(E16*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>349.61677638948368</v>
       </c>
       <c r="T16">
-        <f>IF(I16&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
       <c r="V16" s="2"/>
@@ -1946,11 +1941,11 @@
         <v>8.2268799999999995</v>
       </c>
       <c r="S17">
-        <f>(0.000000000000000138*G17/(1.673534E-24*1.3*0.000000066726*F17*1.8986E+30/(E17*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1280.5918535006856</v>
       </c>
       <c r="T17">
-        <f>IF(I17&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2010,11 +2005,11 @@
         <v>7.5086599999999999</v>
       </c>
       <c r="S18">
-        <f>(0.000000000000000138*G18/(1.673534E-24*1.3*0.000000066726*F18*1.8986E+30/(E18*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>988.21070019970352</v>
       </c>
       <c r="T18">
-        <f>IF(I18&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2074,11 +2069,11 @@
         <v>9.6495599999999992</v>
       </c>
       <c r="S19">
-        <f>(0.000000000000000138*G19/(1.673534E-24*1.3*0.000000066726*F19*1.8986E+30/(E19*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>956.09264119622901</v>
       </c>
       <c r="T19">
-        <f>IF(I19&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2138,11 +2133,11 @@
         <v>7.9077599999999997</v>
       </c>
       <c r="S20">
-        <f>(0.000000000000000138*G20/(1.673534E-24*1.3*0.000000066726*F20*1.8986E+30/(E20*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>742.8583931109747</v>
       </c>
       <c r="T20">
-        <f>IF(I20&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2200,11 +2195,11 @@
         <v>9.5202500000000008</v>
       </c>
       <c r="S21" s="6">
-        <f>(0.000000000000000138*G21/(1.673534E-24*1.3*0.000000066726*F21*1.8986E+30/(E21*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>934.76971602454307</v>
       </c>
       <c r="T21" s="6">
-        <f>IF(I21&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
       <c r="U21" s="7" t="s">
@@ -2267,11 +2262,11 @@
         <v>8.4183900000000005</v>
       </c>
       <c r="S22">
-        <f>(0.000000000000000138*G22/(1.673534E-24*1.3*0.000000066726*F22*1.8986E+30/(E22*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>574.11765847468712</v>
       </c>
       <c r="T22">
-        <f>IF(I22&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2331,11 +2326,11 @@
         <v>7.8097899999999996</v>
       </c>
       <c r="S23">
-        <f>(0.000000000000000138*G23/(1.673534E-24*1.3*0.000000066726*F23*1.8986E+30/(E23*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>668.81110409377118</v>
       </c>
       <c r="T23">
-        <f>IF(I23&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2395,11 +2390,11 @@
         <v>9.2170199999999998</v>
       </c>
       <c r="S24">
-        <f>(0.000000000000000138*G24/(1.673534E-24*1.3*0.000000066726*F24*1.8986E+30/(E24*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1103.5971886171305</v>
       </c>
       <c r="T24">
-        <f>IF(I24&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2456,11 +2451,11 @@
         <v>9.7262599999999999</v>
       </c>
       <c r="S25">
-        <f>(0.000000000000000138*G25/(1.673534E-24*1.3*0.000000066726*F25*1.8986E+30/(E25*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>662.28004924519439</v>
       </c>
       <c r="T25">
-        <f>IF(I25&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2520,11 +2515,11 @@
         <v>7.8311200000000003</v>
       </c>
       <c r="S26">
-        <f>(0.000000000000000138*G26/(1.673534E-24*1.3*0.000000066726*F26*1.8986E+30/(E26*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>3894.9775251994533</v>
       </c>
       <c r="T26">
-        <f>IF(I26&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2584,11 +2579,11 @@
         <v>9.2088699999999992</v>
       </c>
       <c r="S27">
-        <f>(0.000000000000000138*G27/(1.673534E-24*1.3*0.000000066726*F27*1.8986E+30/(E27*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>948.15286253702118</v>
       </c>
       <c r="T27">
-        <f>IF(I27&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -2648,11 +2643,11 @@
         <v>9.8633100000000002</v>
       </c>
       <c r="S28">
-        <f>(0.000000000000000138*G28/(1.673534E-24*1.3*0.000000066726*F28*1.8986E+30/(E28*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>443.85469120292152</v>
       </c>
       <c r="T28">
-        <f>IF(I28&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -2712,11 +2707,11 @@
         <v>8.5839300000000005</v>
       </c>
       <c r="S29">
-        <f>(0.000000000000000138*G29/(1.673534E-24*1.3*0.000000066726*F29*1.8986E+30/(E29*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>570.64953846380126</v>
       </c>
       <c r="T29">
-        <f>IF(I29&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2776,11 +2771,11 @@
         <v>7.5749199999999997</v>
       </c>
       <c r="S30">
-        <f>(0.000000000000000138*G30/(1.673534E-24*1.3*0.000000066726*F30*1.8986E+30/(E30*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>518.80488815900412</v>
       </c>
       <c r="T30">
-        <f>IF(I30&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-7</v>
       </c>
     </row>
@@ -2840,11 +2835,11 @@
         <v>8.23752</v>
       </c>
       <c r="S31">
-        <f>(0.000000000000000138*G31/(1.673534E-24*1.3*0.000000066726*F31*1.8986E+30/(E31*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>99.730517672190274</v>
       </c>
       <c r="T31">
-        <f>IF(I31&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2901,11 +2896,11 @@
         <v>9.7632399999999997</v>
       </c>
       <c r="S32">
-        <f>(0.000000000000000138*G32/(1.673534E-24*1.3*0.000000066726*F32*1.8986E+30/(E32*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>582.97620763372299</v>
       </c>
       <c r="T32">
-        <f>IF(I32&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -2965,11 +2960,11 @@
         <v>9.95702</v>
       </c>
       <c r="S33">
-        <f>(0.000000000000000138*G33/(1.673534E-24*1.3*0.000000066726*F33*1.8986E+30/(E33*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>1492.9814393090719</v>
       </c>
       <c r="T33">
-        <f>IF(I33&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -3029,11 +3024,11 @@
         <v>8.4517299999999995</v>
       </c>
       <c r="S34">
-        <f>(0.000000000000000138*G34/(1.673534E-24*1.3*0.000000066726*F34*1.8986E+30/(E34*7149200000)^2))/100000</f>
+        <f t="shared" si="0"/>
         <v>965.25628287035329</v>
       </c>
       <c r="T34">
-        <f>IF(I34&gt;6800,-7,-5)</f>
+        <f t="shared" si="1"/>
         <v>-5</v>
       </c>
     </row>
@@ -3041,63 +3036,85 @@
       <c r="A35" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="6">
+      <c r="B35" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="19">
         <v>1.4811235</v>
       </c>
-      <c r="D35" s="6">
+      <c r="D35" s="19">
         <v>3.4619999999999998E-2</v>
       </c>
-      <c r="E35" s="6">
+      <c r="E35" s="19">
         <v>1.891</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35" s="19">
         <v>2.88</v>
       </c>
-      <c r="G35" s="6">
+      <c r="G35" s="19">
         <v>4050</v>
       </c>
-      <c r="H35" s="6"/>
-      <c r="I35" s="6"/>
-      <c r="J35" s="6"/>
-      <c r="K35" s="6"/>
-      <c r="L35" s="6"/>
-      <c r="M35" s="6"/>
-      <c r="N35" s="6"/>
-      <c r="O35" s="6"/>
-      <c r="P35" s="6"/>
-      <c r="Q35" s="6"/>
-      <c r="S35" s="6"/>
+      <c r="H35" s="19" t="s">
+        <v>144</v>
+      </c>
+      <c r="I35" s="19">
+        <v>10170</v>
+      </c>
+      <c r="J35" s="19">
+        <v>2.3620000000000001</v>
+      </c>
+      <c r="K35" s="19">
+        <v>2.52</v>
+      </c>
+      <c r="L35" s="19">
+        <v>-0.03</v>
+      </c>
+      <c r="M35" s="19">
+        <v>4.093</v>
+      </c>
+      <c r="N35" s="19">
+        <v>307.85989979999999</v>
+      </c>
+      <c r="O35" s="19">
+        <v>39.9389161</v>
+      </c>
+      <c r="P35" s="19">
+        <v>204.45500000000001</v>
+      </c>
+      <c r="Q35" s="19">
+        <v>7.55</v>
+      </c>
+      <c r="R35" s="19">
+        <v>7.5767499999999997</v>
+      </c>
+      <c r="S35" s="19">
+        <f t="shared" si="0"/>
+        <v>1286.8653667451285</v>
+      </c>
       <c r="T35" s="6"/>
       <c r="U35" s="7" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="H36" s="11"/>
-      <c r="I36" s="17">
+      <c r="I36" s="16">
         <v>7433.197265625</v>
       </c>
-      <c r="J36" s="17"/>
-      <c r="K36" s="11"/>
-      <c r="L36" s="11"/>
-      <c r="M36" s="17"/>
-      <c r="N36" s="17">
+      <c r="J36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16">
         <v>286.97138676797078</v>
       </c>
-      <c r="O36" s="17">
+      <c r="O36" s="16">
         <v>46.868244058307063</v>
       </c>
-      <c r="P36" s="11"/>
-      <c r="Q36" s="17">
+      <c r="Q36" s="16">
         <v>10.382340431213381</v>
       </c>
-      <c r="R36" s="17">
+      <c r="R36" s="16">
         <v>10.382340431213381</v>
       </c>
     </row>
@@ -3154,11 +3171,11 @@
         <v>10.367800000000001</v>
       </c>
       <c r="S37">
-        <f>(0.000000000000000138*G37/(1.673534E-24*1.3*0.000000066726*F37*1.8986E+30/(E37*7149200000)^2))/100000</f>
+        <f t="shared" ref="S37:S63" si="2">(0.000000000000000138*G37/(1.673534E-24*1.3*0.000000066726*F37*1.8986E+30/(E37*7149200000)^2))/100000</f>
         <v>160.76196513632402</v>
       </c>
       <c r="T37">
-        <f>IF(I37&gt;6800,-7,-5)</f>
+        <f t="shared" ref="T37:T63" si="3">IF(I37&gt;6800,-7,-5)</f>
         <v>-7</v>
       </c>
     </row>
@@ -3218,11 +3235,11 @@
         <v>9.6000599999999991</v>
       </c>
       <c r="S38">
-        <f>(0.000000000000000138*G38/(1.673534E-24*1.3*0.000000066726*F38*1.8986E+30/(E38*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>972.96006983022733</v>
       </c>
       <c r="T38">
-        <f>IF(I38&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3282,11 +3299,11 @@
         <v>8.2424300000000006</v>
       </c>
       <c r="S39">
-        <f>(0.000000000000000138*G39/(1.673534E-24*1.3*0.000000066726*F39*1.8986E+30/(E39*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>457.63140850776114</v>
       </c>
       <c r="T39">
-        <f>IF(I39&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3346,11 +3363,11 @@
         <v>8.1740100000000009</v>
       </c>
       <c r="S40">
-        <f>(0.000000000000000138*G40/(1.673534E-24*1.3*0.000000066726*F40*1.8986E+30/(E40*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>789.006338593706</v>
       </c>
       <c r="T40">
-        <f>IF(I40&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3410,11 +3427,11 @@
         <v>9.4290710000000004</v>
       </c>
       <c r="S41" s="6">
-        <f>(0.000000000000000138*G41/(1.673534E-24*1.3*0.000000066726*F41*1.8986E+30/(E41*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>56.120615203365361</v>
       </c>
       <c r="T41" s="6">
-        <f>IF(I41&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
       <c r="U41" s="7" t="s">
@@ -3477,11 +3494,11 @@
         <v>9.4135299999999997</v>
       </c>
       <c r="S42">
-        <f>(0.000000000000000138*G42/(1.673534E-24*1.3*0.000000066726*F42*1.8986E+30/(E42*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1175.9460676296278</v>
       </c>
       <c r="T42">
-        <f>IF(I42&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3538,11 +3555,11 @@
         <v>9.3678899999999992</v>
       </c>
       <c r="S43">
-        <f>(0.000000000000000138*G43/(1.673534E-24*1.3*0.000000066726*F43*1.8986E+30/(E43*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1399.2265914107247</v>
       </c>
       <c r="T43">
-        <f>IF(I43&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3599,11 +3616,11 @@
         <v>9.3503900000000009</v>
       </c>
       <c r="S44">
-        <f>(0.000000000000000138*G44/(1.673534E-24*1.3*0.000000066726*F44*1.8986E+30/(E44*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>353.31388599481477</v>
       </c>
       <c r="T44">
-        <f>IF(I44&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3663,11 +3680,11 @@
         <v>9.1879500000000007</v>
       </c>
       <c r="S45">
-        <f>(0.000000000000000138*G45/(1.673534E-24*1.3*0.000000066726*F45*1.8986E+30/(E45*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>882.20971786077962</v>
       </c>
       <c r="T45">
-        <f>IF(I45&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3727,11 +3744,11 @@
         <v>7.9756099999999996</v>
       </c>
       <c r="S46">
-        <f>(0.000000000000000138*G46/(1.673534E-24*1.3*0.000000066726*F46*1.8986E+30/(E46*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>431.57254486096394</v>
       </c>
       <c r="T46">
-        <f>IF(I46&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3791,11 +3808,11 @@
         <v>8.8952899999999993</v>
       </c>
       <c r="S47">
-        <f>(0.000000000000000138*G47/(1.673534E-24*1.3*0.000000066726*F47*1.8986E+30/(E47*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>974.78820571370204</v>
       </c>
       <c r="T47">
-        <f>IF(I47&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -3855,11 +3872,11 @@
         <v>9.5843900000000009</v>
       </c>
       <c r="S48">
-        <f>(0.000000000000000138*G48/(1.673534E-24*1.3*0.000000066726*F48*1.8986E+30/(E48*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1460.8182255852041</v>
       </c>
       <c r="T48">
-        <f>IF(I48&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3916,11 +3933,11 @@
         <v>9.6598100000000002</v>
       </c>
       <c r="S49">
-        <f>(0.000000000000000138*G49/(1.673534E-24*1.3*0.000000066726*F49*1.8986E+30/(E49*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1324.5165539963698</v>
       </c>
       <c r="T49">
-        <f>IF(I49&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -3977,11 +3994,11 @@
         <v>9.7596699999999998</v>
       </c>
       <c r="S50">
-        <f>(0.000000000000000138*G50/(1.673534E-24*1.3*0.000000066726*F50*1.8986E+30/(E50*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>55.915145726222889</v>
       </c>
       <c r="T50">
-        <f>IF(I50&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -4038,11 +4055,11 @@
         <v>8.9365100000000002</v>
       </c>
       <c r="S51">
-        <f>(0.000000000000000138*G51/(1.673534E-24*1.3*0.000000066726*F51*1.8986E+30/(E51*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>77.040187113891676</v>
       </c>
       <c r="T51">
-        <f>IF(I51&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4099,11 +4116,11 @@
         <v>9.4724400000000006</v>
       </c>
       <c r="S52">
-        <f>(0.000000000000000138*G52/(1.673534E-24*1.3*0.000000066726*F52*1.8986E+30/(E52*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>83.670803141549356</v>
       </c>
       <c r="T52">
-        <f>IF(I52&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-7</v>
       </c>
     </row>
@@ -4160,11 +4177,11 @@
         <v>7.4165299999999998</v>
       </c>
       <c r="S53">
-        <f>(0.000000000000000138*G53/(1.673534E-24*1.3*0.000000066726*F53*1.8986E+30/(E53*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>777.64358420307099</v>
       </c>
       <c r="T53">
-        <f>IF(I53&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4224,11 +4241,11 @@
         <v>9.7777600000000007</v>
       </c>
       <c r="S54">
-        <f>(0.000000000000000138*G54/(1.673534E-24*1.3*0.000000066726*F54*1.8986E+30/(E54*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>755.33252275944176</v>
       </c>
       <c r="T54">
-        <f>IF(I54&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4285,11 +4302,11 @@
         <v>9.641</v>
       </c>
       <c r="S55">
-        <f>(0.000000000000000138*G55/(1.673534E-24*1.3*0.000000066726*F55*1.8986E+30/(E55*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>318.17832033985127</v>
       </c>
       <c r="T55">
-        <f>IF(I55&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4349,11 +4366,11 @@
         <v>9.0746900000000004</v>
       </c>
       <c r="S56">
-        <f>(0.000000000000000138*G56/(1.673534E-24*1.3*0.000000066726*F56*1.8986E+30/(E56*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>36.149567272802649</v>
       </c>
       <c r="T56">
-        <f>IF(I56&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4413,11 +4430,11 @@
         <v>9.8465900000000008</v>
       </c>
       <c r="S57">
-        <f>(0.000000000000000138*G57/(1.673534E-24*1.3*0.000000066726*F57*1.8986E+30/(E57*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>224.58825733889913</v>
       </c>
       <c r="T57">
-        <f>IF(I57&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4474,11 +4491,11 @@
         <v>9.6080000000000005</v>
       </c>
       <c r="S58">
-        <f>(0.000000000000000138*G58/(1.673534E-24*1.3*0.000000066726*F58*1.8986E+30/(E58*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1039.84328949877</v>
       </c>
       <c r="T58">
-        <f>IF(I58&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4538,11 +4555,11 @@
         <v>9.9823299999999993</v>
       </c>
       <c r="S59">
-        <f>(0.000000000000000138*G59/(1.673534E-24*1.3*0.000000066726*F59*1.8986E+30/(E59*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>1107.9861243219782</v>
       </c>
       <c r="T59">
-        <f>IF(I59&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4599,11 +4616,11 @@
         <v>9.7295700000000007</v>
       </c>
       <c r="S60">
-        <f>(0.000000000000000138*G60/(1.673534E-24*1.3*0.000000066726*F60*1.8986E+30/(E60*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>487.59044264912109</v>
       </c>
       <c r="T60">
-        <f>IF(I60&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4663,11 +4680,11 @@
         <v>8.8910300000000007</v>
       </c>
       <c r="S61">
-        <f>(0.000000000000000138*G61/(1.673534E-24*1.3*0.000000066726*F61*1.8986E+30/(E61*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>795.95548671567838</v>
       </c>
       <c r="T61">
-        <f>IF(I61&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4727,11 +4744,11 @@
         <v>9.6608199999999993</v>
       </c>
       <c r="S62">
-        <f>(0.000000000000000138*G62/(1.673534E-24*1.3*0.000000066726*F62*1.8986E+30/(E62*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>355.42536038318485</v>
       </c>
       <c r="T62">
-        <f>IF(I62&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
@@ -4791,45 +4808,43 @@
         <v>8.9943600000000004</v>
       </c>
       <c r="S63">
-        <f>(0.000000000000000138*G63/(1.673534E-24*1.3*0.000000066726*F63*1.8986E+30/(E63*7149200000)^2))/100000</f>
+        <f t="shared" si="2"/>
         <v>267.77715667890726</v>
       </c>
       <c r="T63">
-        <f>IF(I63&gt;6800,-7,-5)</f>
+        <f t="shared" si="3"/>
         <v>-5</v>
       </c>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A64" s="12" t="s">
+      <c r="A64" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="H64" s="11"/>
-      <c r="I64" s="17">
+      <c r="I64" s="16">
         <v>6161.02294921875</v>
       </c>
-      <c r="J64" s="17">
+      <c r="J64" s="16">
         <v>1.7061723470687871</v>
       </c>
-      <c r="K64" s="11">
+      <c r="K64">
         <v>1.3463604</v>
       </c>
-      <c r="L64" s="11"/>
-      <c r="M64" s="17">
+      <c r="M64" s="16">
         <v>3.9825000762939449</v>
       </c>
-      <c r="N64" s="11">
+      <c r="N64">
         <v>268.30433503422898</v>
       </c>
-      <c r="O64" s="17">
+      <c r="O64" s="16">
         <v>37.211736733677057</v>
       </c>
-      <c r="P64" s="11">
+      <c r="P64">
         <v>496.26729999999998</v>
       </c>
-      <c r="Q64" s="17">
+      <c r="Q64" s="16">
         <v>11.469913482666019</v>
       </c>
-      <c r="R64" s="17">
+      <c r="R64" s="16">
         <v>11.469913482666019</v>
       </c>
     </row>
@@ -4859,7 +4874,7 @@
         <v>11.4986</v>
       </c>
       <c r="T65">
-        <f>IF(I65&gt;6800,-7,-5)</f>
+        <f t="shared" ref="T65:T85" si="4">IF(I65&gt;6800,-7,-5)</f>
         <v>-5</v>
       </c>
     </row>
@@ -4919,11 +4934,11 @@
         <v>9.8670799999999996</v>
       </c>
       <c r="S66">
-        <f>(0.000000000000000138*G66/(1.673534E-24*1.3*0.000000066726*F66*1.8986E+30/(E66*7149200000)^2))/100000</f>
+        <f t="shared" ref="S66:S85" si="5">(0.000000000000000138*G66/(1.673534E-24*1.3*0.000000066726*F66*1.8986E+30/(E66*7149200000)^2))/100000</f>
         <v>2057.1154637812851</v>
       </c>
       <c r="T66">
-        <f>IF(I66&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -4983,11 +4998,11 @@
         <v>9.8192900000000005</v>
       </c>
       <c r="S67">
-        <f>(0.000000000000000138*G67/(1.673534E-24*1.3*0.000000066726*F67*1.8986E+30/(E67*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>621.55661806820979</v>
       </c>
       <c r="T67">
-        <f>IF(I67&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5044,11 +5059,11 @@
         <v>9.6464700000000008</v>
       </c>
       <c r="S68">
-        <f>(0.000000000000000138*G68/(1.673534E-24*1.3*0.000000066726*F68*1.8986E+30/(E68*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>103.20465157174387</v>
       </c>
       <c r="T68">
-        <f>IF(I68&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5108,11 +5123,11 @@
         <v>9.2569999999999997</v>
       </c>
       <c r="S69">
-        <f>(0.000000000000000138*G69/(1.673534E-24*1.3*0.000000066726*F69*1.8986E+30/(E69*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>1277.1766379712274</v>
       </c>
       <c r="T69">
-        <f>IF(I69&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5172,11 +5187,11 @@
         <v>9.9122599999999998</v>
       </c>
       <c r="S70">
-        <f>(0.000000000000000138*G70/(1.673534E-24*1.3*0.000000066726*F70*1.8986E+30/(E70*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>1247.4798366438731</v>
       </c>
       <c r="T70">
-        <f>IF(I70&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-7</v>
       </c>
     </row>
@@ -5236,11 +5251,11 @@
         <v>9.1661699999999993</v>
       </c>
       <c r="S71">
-        <f>(0.000000000000000138*G71/(1.673534E-24*1.3*0.000000066726*F71*1.8986E+30/(E71*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>93.704022194109143</v>
       </c>
       <c r="T71">
-        <f>IF(I71&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5298,11 +5313,11 @@
         <v>6.5536899999999996</v>
       </c>
       <c r="S72" s="8">
-        <f>(0.000000000000000138*G72/(1.673534E-24*1.3*0.000000066726*F72*1.8986E+30/(E72*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>1130.2166328238993</v>
       </c>
       <c r="T72" s="6">
-        <f>IF(I72&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-7</v>
       </c>
       <c r="U72" s="7" t="s">
@@ -5365,11 +5380,11 @@
         <v>8.0700400000000005</v>
       </c>
       <c r="S73">
-        <f>(0.000000000000000138*G73/(1.673534E-24*1.3*0.000000066726*F73*1.8986E+30/(E73*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>863.09804630713359</v>
       </c>
       <c r="T73">
-        <f>IF(I73&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-7</v>
       </c>
     </row>
@@ -5429,11 +5444,11 @@
         <v>9.20974</v>
       </c>
       <c r="S74">
-        <f>(0.000000000000000138*G74/(1.673534E-24*1.3*0.000000066726*F74*1.8986E+30/(E74*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>140.68549179703928</v>
       </c>
       <c r="T74">
-        <f>IF(I74&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5493,11 +5508,11 @@
         <v>9.4846599999999999</v>
       </c>
       <c r="S75" s="6">
-        <f>(0.000000000000000138*G75/(1.673534E-24*1.3*0.000000066726*F75*1.8986E+30/(E75*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>955.72600175951948</v>
       </c>
       <c r="T75" s="6">
-        <f>IF(I75&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
       <c r="U75" s="7" t="s">
@@ -5557,11 +5572,11 @@
         <v>9.3767099999999992</v>
       </c>
       <c r="S76">
-        <f>(0.000000000000000138*G76/(1.673534E-24*1.3*0.000000066726*F76*1.8986E+30/(E76*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>701.18164217622461</v>
       </c>
       <c r="T76">
-        <f>IF(I76&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5621,11 +5636,11 @@
         <v>9.5723000000000003</v>
       </c>
       <c r="S77">
-        <f>(0.000000000000000138*G77/(1.673534E-24*1.3*0.000000066726*F77*1.8986E+30/(E77*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>1226.0598654781754</v>
       </c>
       <c r="T77">
-        <f>IF(I77&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5685,11 +5700,11 @@
         <v>9.3950700000000005</v>
       </c>
       <c r="S78">
-        <f>(0.000000000000000138*G78/(1.673534E-24*1.3*0.000000066726*F78*1.8986E+30/(E78*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>2192.2225820487197</v>
       </c>
       <c r="T78">
-        <f>IF(I78&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5749,11 +5764,11 @@
         <v>9.9720200000000006</v>
       </c>
       <c r="S79">
-        <f>(0.000000000000000138*G79/(1.673534E-24*1.3*0.000000066726*F79*1.8986E+30/(E79*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>1209.5375438309629</v>
       </c>
       <c r="T79">
-        <f>IF(I79&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5813,11 +5828,11 @@
         <v>9.6124899999999993</v>
       </c>
       <c r="S80">
-        <f>(0.000000000000000138*G80/(1.673534E-24*1.3*0.000000066726*F80*1.8986E+30/(E80*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>136.24063220140397</v>
       </c>
       <c r="T80">
-        <f>IF(I80&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
@@ -5846,10 +5861,10 @@
       <c r="H81" t="s">
         <v>127</v>
       </c>
-      <c r="I81" s="16">
+      <c r="I81" s="15">
         <v>6480</v>
       </c>
-      <c r="J81" s="16">
+      <c r="J81" s="15">
         <v>2.1</v>
       </c>
       <c r="K81">
@@ -5858,38 +5873,38 @@
       <c r="L81">
         <v>0.12</v>
       </c>
-      <c r="M81" s="16">
+      <c r="M81" s="15">
         <v>3.96</v>
       </c>
-      <c r="N81" s="16">
+      <c r="N81" s="15">
         <v>72.660591600000004</v>
       </c>
-      <c r="O81" s="16">
+      <c r="O81" s="15">
         <v>1.8938364999999999</v>
       </c>
       <c r="P81">
         <v>275.66399999999999</v>
       </c>
-      <c r="Q81" s="16">
+      <c r="Q81" s="15">
         <v>10.073</v>
       </c>
-      <c r="R81" s="20">
+      <c r="R81" s="18">
         <v>9.8979599999999994</v>
       </c>
       <c r="S81">
-        <f>(0.000000000000000138*G81/(1.673534E-24*1.3*0.000000066726*F81*1.8986E+30/(E81*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>1257.117296864338</v>
       </c>
       <c r="T81">
-        <f>IF(I81&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A82" s="13" t="s">
+      <c r="A82" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B82" s="16" t="s">
+      <c r="B82" s="15" t="s">
         <v>20</v>
       </c>
       <c r="C82">
@@ -5910,10 +5925,10 @@
       <c r="H82" t="s">
         <v>54</v>
       </c>
-      <c r="I82" s="16">
+      <c r="I82" s="15">
         <v>6170</v>
       </c>
-      <c r="J82" s="16">
+      <c r="J82" s="15">
         <v>1.48</v>
       </c>
       <c r="K82">
@@ -5922,35 +5937,35 @@
       <c r="L82">
         <v>0.26</v>
       </c>
-      <c r="M82" s="16">
+      <c r="M82" s="15">
         <v>4.2699999999999996</v>
       </c>
-      <c r="N82" s="16">
+      <c r="N82" s="15">
         <v>313.78323929999999</v>
       </c>
-      <c r="O82" s="16">
+      <c r="O82" s="15">
         <v>-34.135751200000001</v>
       </c>
       <c r="P82">
         <v>211.21100000000001</v>
       </c>
-      <c r="Q82" s="16">
+      <c r="Q82" s="15">
         <v>10.051</v>
       </c>
-      <c r="R82" s="20">
+      <c r="R82" s="18">
         <v>10.028499999999999</v>
       </c>
       <c r="S82">
-        <f>(0.000000000000000138*G82/(1.673534E-24*1.3*0.000000066726*F82*1.8986E+30/(E82*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>2049.4439875099679</v>
       </c>
       <c r="T82">
-        <f>IF(I82&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A83" s="13" t="s">
+      <c r="A83" s="12" t="s">
         <v>133</v>
       </c>
       <c r="B83" t="s">
@@ -5974,10 +5989,10 @@
       <c r="H83" t="s">
         <v>134</v>
       </c>
-      <c r="I83" s="16">
+      <c r="I83" s="15">
         <v>5830</v>
       </c>
-      <c r="J83" s="16">
+      <c r="J83" s="15">
         <v>1.23</v>
       </c>
       <c r="K83">
@@ -5986,35 +6001,35 @@
       <c r="L83">
         <v>0.14000000000000001</v>
       </c>
-      <c r="M83" s="16">
+      <c r="M83" s="15">
         <v>4.3600000000000003</v>
       </c>
-      <c r="N83" s="16">
+      <c r="N83" s="15">
         <v>337.45782430000003</v>
       </c>
-      <c r="O83" s="16">
+      <c r="O83" s="15">
         <v>-48.003098799999997</v>
       </c>
       <c r="P83">
         <v>137.54400000000001</v>
       </c>
-      <c r="Q83" s="16">
+      <c r="Q83" s="15">
         <v>10.092000000000001</v>
       </c>
-      <c r="R83" s="20">
+      <c r="R83" s="18">
         <v>9.9369700000000005</v>
       </c>
       <c r="S83">
-        <f>(0.000000000000000138*G83/(1.673534E-24*1.3*0.000000066726*F83*1.8986E+30/(E83*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>422.11900227636102</v>
       </c>
       <c r="T83">
-        <f>IF(I83&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
     <row r="84" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A84" s="13" t="s">
+      <c r="A84" s="12" t="s">
         <v>79</v>
       </c>
       <c r="B84" t="s">
@@ -6035,50 +6050,50 @@
       <c r="G84">
         <v>1480</v>
       </c>
-      <c r="H84" s="11" t="s">
+      <c r="H84" t="s">
         <v>54</v>
       </c>
-      <c r="I84" s="18">
+      <c r="I84" s="15">
         <v>6150</v>
       </c>
-      <c r="J84" s="18">
+      <c r="J84" s="15">
         <v>1.64</v>
       </c>
-      <c r="K84" s="11">
+      <c r="K84">
         <v>1.21</v>
       </c>
-      <c r="L84" s="11">
+      <c r="L84">
         <v>0.21</v>
       </c>
-      <c r="M84" s="18">
+      <c r="M84" s="15">
         <v>4.3</v>
       </c>
-      <c r="N84" s="18">
+      <c r="N84" s="15">
         <v>39.897668899999999</v>
       </c>
-      <c r="O84" s="18">
+      <c r="O84" s="15">
         <v>-50.008193400000003</v>
       </c>
-      <c r="P84" s="11">
+      <c r="P84">
         <v>158.66</v>
       </c>
-      <c r="Q84" s="18">
+      <c r="Q84" s="15">
         <v>9.4749999999999996</v>
       </c>
-      <c r="R84" s="18">
+      <c r="R84" s="15">
         <v>9.3251000000000008</v>
       </c>
       <c r="S84">
-        <f>(0.000000000000000138*G84/(1.673534E-24*1.3*0.000000066726*F84*1.8986E+30/(E84*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>162.15983922320817</v>
       </c>
       <c r="T84">
-        <f>IF(I84&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
     <row r="85" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="A85" s="13" t="s">
+      <c r="A85" s="12" t="s">
         <v>107</v>
       </c>
       <c r="B85" t="s">
@@ -6099,60 +6114,50 @@
       <c r="G85">
         <v>1729</v>
       </c>
-      <c r="H85" s="11" t="s">
+      <c r="H85" t="s">
         <v>108</v>
       </c>
-      <c r="I85" s="19">
+      <c r="I85" s="17">
         <v>6429</v>
       </c>
-      <c r="J85" s="19">
+      <c r="J85" s="17">
         <v>1.54</v>
       </c>
-      <c r="K85" s="11">
+      <c r="K85">
         <v>0.57999999999999996</v>
       </c>
-      <c r="L85" s="11">
+      <c r="L85">
         <v>-0.18</v>
       </c>
-      <c r="M85" s="19">
+      <c r="M85" s="17">
         <v>3.95</v>
       </c>
-      <c r="N85" s="11">
+      <c r="N85">
         <v>65.469581399999996</v>
       </c>
-      <c r="O85" s="19">
+      <c r="O85" s="17">
         <v>57.817209499999997</v>
       </c>
-      <c r="P85" s="11">
+      <c r="P85">
         <v>213.053</v>
       </c>
-      <c r="Q85" s="19">
+      <c r="Q85" s="17">
         <v>9.8539999999999992</v>
       </c>
-      <c r="R85" s="19">
+      <c r="R85" s="17">
         <v>9.7388899999999996</v>
       </c>
       <c r="S85">
-        <f>(0.000000000000000138*G85/(1.673534E-24*1.3*0.000000066726*F85*1.8986E+30/(E85*7149200000)^2))/100000</f>
+        <f t="shared" si="5"/>
         <v>120.66830436099001</v>
       </c>
       <c r="T85">
-        <f>IF(I85&gt;6800,-7,-5)</f>
+        <f t="shared" si="4"/>
         <v>-5</v>
       </c>
     </row>
     <row r="86" spans="1:20" x14ac:dyDescent="0.2">
-      <c r="H86" s="11"/>
-      <c r="I86" s="11"/>
-      <c r="J86" s="11"/>
-      <c r="K86" s="11"/>
-      <c r="L86" s="11"/>
-      <c r="M86" s="11"/>
-      <c r="N86" s="11"/>
-      <c r="O86" s="11"/>
-      <c r="P86" s="11"/>
-      <c r="Q86" s="11"/>
-      <c r="R86" s="11"/>
+      <c r="R86"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U79" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
added gaiahelpers and roland call stars
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55D4D5BB-BFFC-0C4C-988C-A73FCF734FFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0968ED-5547-EE4A-A5BC-D62327CC2110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22040" yWindow="820" windowWidth="33600" windowHeight="25500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3080" yWindow="860" windowWidth="30820" windowHeight="25500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="154">
   <si>
     <t>#pl_name</t>
   </si>
@@ -471,6 +471,33 @@
   </si>
   <si>
     <t>B9.5-A0</t>
+  </si>
+  <si>
+    <t>V_MAG</t>
+  </si>
+  <si>
+    <t>B_MAG</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>4236349174325957504 b</t>
+  </si>
+  <si>
+    <t>DWARF</t>
+  </si>
+  <si>
+    <t>4186786759262834816 b</t>
+  </si>
+  <si>
+    <t>GIANT</t>
+  </si>
+  <si>
+    <t>4999199962400320128 b</t>
+  </si>
+  <si>
+    <t>4760966338470589184 b</t>
   </si>
 </sst>
 </file>
@@ -480,7 +507,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000_ "/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -502,8 +529,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -540,8 +573,14 @@
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -590,13 +629,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -647,6 +701,28 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -924,14 +1000,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH86"/>
+  <dimension ref="A1:BH89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.6640625" customWidth="1"/>
     <col min="3" max="4" width="12.5"/>
     <col min="5" max="6" width="11.33203125"/>
-    <col min="7" max="10" width="8.1640625"/>
+    <col min="7" max="8" width="8.1640625"/>
+    <col min="9" max="9" width="9.6640625" style="21" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.1640625"/>
     <col min="11" max="11" width="9.1640625"/>
     <col min="14" max="15" width="12.5"/>
     <col min="16" max="16" width="9"/>
@@ -983,7 +1061,7 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="21" t="s">
         <v>8</v>
       </c>
       <c r="J1" t="s">
@@ -1021,13 +1099,22 @@
       </c>
       <c r="U1" s="4" t="s">
         <v>136</v>
+      </c>
+      <c r="V1" s="20" t="s">
+        <v>145</v>
+      </c>
+      <c r="W1" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="X1" s="20" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="I2" s="16">
+      <c r="I2" s="22">
         <v>4907.77490234375</v>
       </c>
       <c r="J2" s="16"/>
@@ -1073,7 +1160,7 @@
       <c r="H3" t="s">
         <v>27</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="21">
         <v>5980</v>
       </c>
       <c r="J3">
@@ -1140,7 +1227,7 @@
       <c r="H4" t="s">
         <v>125</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="21">
         <v>6600</v>
       </c>
       <c r="J4">
@@ -1207,7 +1294,7 @@
       <c r="H5" t="s">
         <v>54</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="21">
         <v>6380</v>
       </c>
       <c r="J5">
@@ -1274,7 +1361,7 @@
       <c r="H6" t="s">
         <v>94</v>
       </c>
-      <c r="I6">
+      <c r="I6" s="21">
         <v>5302</v>
       </c>
       <c r="J6">
@@ -1321,7 +1408,7 @@
         <v>140</v>
       </c>
       <c r="B7" s="14"/>
-      <c r="I7" s="16">
+      <c r="I7" s="22">
         <v>6245.11328125</v>
       </c>
       <c r="J7" s="16">
@@ -1371,7 +1458,7 @@
       <c r="G8">
         <v>1772</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="21">
         <v>6212</v>
       </c>
       <c r="J8">
@@ -1435,7 +1522,7 @@
       <c r="G9">
         <v>1930</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="21">
         <v>7394</v>
       </c>
       <c r="J9">
@@ -1478,7 +1565,7 @@
       <c r="A10" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="22">
         <v>6424.27685546875</v>
       </c>
       <c r="J10" s="16">
@@ -1520,7 +1607,7 @@
       <c r="G11">
         <v>2562</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="21">
         <v>8450</v>
       </c>
       <c r="J11">
@@ -1587,7 +1674,7 @@
       <c r="H12" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="2">
+      <c r="I12" s="23">
         <v>5742</v>
       </c>
       <c r="J12" s="2">
@@ -1651,7 +1738,7 @@
       <c r="H13" t="s">
         <v>31</v>
       </c>
-      <c r="I13">
+      <c r="I13" s="21">
         <v>5521</v>
       </c>
       <c r="J13">
@@ -1715,7 +1802,7 @@
       <c r="H14" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="I14" s="2">
+      <c r="I14" s="23">
         <v>6179</v>
       </c>
       <c r="J14" s="2">
@@ -1782,7 +1869,7 @@
       <c r="H15" t="s">
         <v>43</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="21">
         <v>6310</v>
       </c>
       <c r="J15">
@@ -1846,7 +1933,7 @@
       <c r="H16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I16" s="2">
+      <c r="I16" s="23">
         <v>5052</v>
       </c>
       <c r="J16" s="2">
@@ -1910,7 +1997,7 @@
       <c r="G17">
         <v>2132</v>
       </c>
-      <c r="I17">
+      <c r="I17" s="21">
         <v>6272</v>
       </c>
       <c r="J17">
@@ -1974,7 +2061,7 @@
       <c r="H18" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I18" s="2">
+      <c r="I18" s="23">
         <v>6091</v>
       </c>
       <c r="J18" s="2">
@@ -2038,7 +2125,7 @@
       <c r="H19" t="s">
         <v>94</v>
       </c>
-      <c r="I19">
+      <c r="I19" s="21">
         <v>5540</v>
       </c>
       <c r="J19">
@@ -2102,7 +2189,7 @@
       <c r="H20" t="s">
         <v>45</v>
       </c>
-      <c r="I20">
+      <c r="I20" s="21">
         <v>5080</v>
       </c>
       <c r="J20">
@@ -2164,7 +2251,7 @@
         <v>2061</v>
       </c>
       <c r="H21" s="6"/>
-      <c r="I21" s="6">
+      <c r="I21" s="24">
         <v>6801</v>
       </c>
       <c r="J21" s="6">
@@ -2231,7 +2318,7 @@
       <c r="H22" t="s">
         <v>54</v>
       </c>
-      <c r="I22">
+      <c r="I22" s="21">
         <v>6128</v>
       </c>
       <c r="J22">
@@ -2295,7 +2382,7 @@
       <c r="H23" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="I23" s="2">
+      <c r="I23" s="23">
         <v>5392</v>
       </c>
       <c r="J23" s="2">
@@ -2359,7 +2446,7 @@
       <c r="H24" t="s">
         <v>33</v>
       </c>
-      <c r="I24">
+      <c r="I24" s="21">
         <v>5576</v>
       </c>
       <c r="J24">
@@ -2420,7 +2507,7 @@
       <c r="G25">
         <v>1030</v>
       </c>
-      <c r="I25">
+      <c r="I25" s="21">
         <v>6154</v>
       </c>
       <c r="J25">
@@ -2484,7 +2571,7 @@
       <c r="H26" t="s">
         <v>37</v>
       </c>
-      <c r="I26">
+      <c r="I26" s="21">
         <v>5375</v>
       </c>
       <c r="J26">
@@ -2548,7 +2635,7 @@
       <c r="H27" t="s">
         <v>41</v>
       </c>
-      <c r="I27">
+      <c r="I27" s="21">
         <v>7454</v>
       </c>
       <c r="J27">
@@ -2612,7 +2699,7 @@
       <c r="H28" t="s">
         <v>110</v>
       </c>
-      <c r="I28">
+      <c r="I28" s="21">
         <v>7500</v>
       </c>
       <c r="J28">
@@ -2676,7 +2763,7 @@
       <c r="H29" t="s">
         <v>54</v>
       </c>
-      <c r="I29">
+      <c r="I29" s="21">
         <v>6327</v>
       </c>
       <c r="J29">
@@ -2740,7 +2827,7 @@
       <c r="H30" t="s">
         <v>24</v>
       </c>
-      <c r="I30">
+      <c r="I30" s="21">
         <v>8720</v>
       </c>
       <c r="J30">
@@ -2804,7 +2891,7 @@
       <c r="H31" t="s">
         <v>52</v>
       </c>
-      <c r="I31">
+      <c r="I31" s="21">
         <v>6426</v>
       </c>
       <c r="J31">
@@ -2865,7 +2952,7 @@
       <c r="G32">
         <v>1816</v>
       </c>
-      <c r="I32">
+      <c r="I32" s="21">
         <v>6304</v>
       </c>
       <c r="J32">
@@ -2929,7 +3016,7 @@
       <c r="H33" t="s">
         <v>56</v>
       </c>
-      <c r="I33">
+      <c r="I33" s="21">
         <v>6206</v>
       </c>
       <c r="J33">
@@ -2993,7 +3080,7 @@
       <c r="H34" t="s">
         <v>56</v>
       </c>
-      <c r="I34">
+      <c r="I34" s="21">
         <v>6768</v>
       </c>
       <c r="J34">
@@ -3057,8 +3144,8 @@
       <c r="H35" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="I35" s="19">
-        <v>10170</v>
+      <c r="I35" s="25">
+        <v>10170.1</v>
       </c>
       <c r="J35" s="19">
         <v>2.3620000000000001</v>
@@ -3100,7 +3187,7 @@
       <c r="A36" s="11" t="s">
         <v>142</v>
       </c>
-      <c r="I36" s="16">
+      <c r="I36" s="22">
         <v>7433.197265625</v>
       </c>
       <c r="J36" s="16"/>
@@ -3140,7 +3227,7 @@
       <c r="G37">
         <v>2550</v>
       </c>
-      <c r="I37">
+      <c r="I37" s="21">
         <v>7650</v>
       </c>
       <c r="J37">
@@ -3204,7 +3291,7 @@
       <c r="H38" t="s">
         <v>99</v>
       </c>
-      <c r="I38">
+      <c r="I38" s="21">
         <v>5443</v>
       </c>
       <c r="J38">
@@ -3268,7 +3355,7 @@
       <c r="H39" t="s">
         <v>49</v>
       </c>
-      <c r="I39">
+      <c r="I39" s="21">
         <v>7490</v>
       </c>
       <c r="J39">
@@ -3332,7 +3419,7 @@
       <c r="H40" t="s">
         <v>47</v>
       </c>
-      <c r="I40">
+      <c r="I40" s="21">
         <v>7800</v>
       </c>
       <c r="J40">
@@ -3396,7 +3483,7 @@
       <c r="H41" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I41" s="6">
+      <c r="I41" s="24">
         <v>5756</v>
       </c>
       <c r="J41" s="6">
@@ -3463,7 +3550,7 @@
       <c r="H42" t="s">
         <v>43</v>
       </c>
-      <c r="I42">
+      <c r="I42" s="21">
         <v>5962.7</v>
       </c>
       <c r="J42">
@@ -3524,7 +3611,7 @@
       <c r="G43">
         <v>843</v>
       </c>
-      <c r="I43">
+      <c r="I43" s="21">
         <v>5770</v>
       </c>
       <c r="J43">
@@ -3585,7 +3672,7 @@
       <c r="G44">
         <v>1679</v>
       </c>
-      <c r="I44">
+      <c r="I44" s="21">
         <v>6274</v>
       </c>
       <c r="J44">
@@ -3649,7 +3736,7 @@
       <c r="H45" t="s">
         <v>70</v>
       </c>
-      <c r="I45">
+      <c r="I45" s="21">
         <v>6117</v>
       </c>
       <c r="J45">
@@ -3713,7 +3800,7 @@
       <c r="H46" t="s">
         <v>35</v>
       </c>
-      <c r="I46">
+      <c r="I46" s="21">
         <v>7690</v>
       </c>
       <c r="J46">
@@ -3777,7 +3864,7 @@
       <c r="H47" t="s">
         <v>61</v>
       </c>
-      <c r="I47">
+      <c r="I47" s="21">
         <v>7300</v>
       </c>
       <c r="J47">
@@ -3841,7 +3928,7 @@
       <c r="H48" t="s">
         <v>56</v>
       </c>
-      <c r="I48">
+      <c r="I48" s="21">
         <v>5991</v>
       </c>
       <c r="J48">
@@ -3902,7 +3989,7 @@
       <c r="G49">
         <v>1199.55</v>
       </c>
-      <c r="I49">
+      <c r="I49" s="21">
         <v>6039</v>
       </c>
       <c r="J49">
@@ -3963,7 +4050,7 @@
       <c r="G50">
         <v>1221.3900000000001</v>
       </c>
-      <c r="I50">
+      <c r="I50" s="21">
         <v>7130</v>
       </c>
       <c r="J50">
@@ -4024,7 +4111,7 @@
       <c r="G51">
         <v>1363.43</v>
       </c>
-      <c r="I51">
+      <c r="I51" s="21">
         <v>6200</v>
       </c>
       <c r="J51">
@@ -4085,7 +4172,7 @@
       <c r="G52">
         <v>1595</v>
       </c>
-      <c r="I52">
+      <c r="I52" s="21">
         <v>7360</v>
       </c>
       <c r="J52">
@@ -4146,7 +4233,7 @@
       <c r="G53">
         <v>1027</v>
       </c>
-      <c r="I53">
+      <c r="I53" s="21">
         <v>6095</v>
       </c>
       <c r="J53">
@@ -4210,7 +4297,7 @@
       <c r="H54" t="s">
         <v>116</v>
       </c>
-      <c r="I54">
+      <c r="I54" s="21">
         <v>5291</v>
       </c>
       <c r="J54">
@@ -4271,7 +4358,7 @@
       <c r="G55">
         <v>1655</v>
       </c>
-      <c r="I55">
+      <c r="I55" s="21">
         <v>4896</v>
       </c>
       <c r="J55">
@@ -4335,7 +4422,7 @@
       <c r="H56" t="s">
         <v>56</v>
       </c>
-      <c r="I56">
+      <c r="I56" s="21">
         <v>6264</v>
       </c>
       <c r="J56">
@@ -4399,7 +4486,7 @@
       <c r="H57" t="s">
         <v>120</v>
       </c>
-      <c r="I57">
+      <c r="I57" s="21">
         <v>5735</v>
       </c>
       <c r="J57">
@@ -4460,7 +4547,7 @@
       <c r="G58">
         <v>1180</v>
       </c>
-      <c r="I58">
+      <c r="I58" s="21">
         <v>5808</v>
       </c>
       <c r="J58">
@@ -4524,7 +4611,7 @@
       <c r="H59" t="s">
         <v>130</v>
       </c>
-      <c r="I59">
+      <c r="I59" s="21">
         <v>6000</v>
       </c>
       <c r="J59">
@@ -4585,7 +4672,7 @@
       <c r="G60">
         <v>1439</v>
       </c>
-      <c r="I60">
+      <c r="I60" s="21">
         <v>6110</v>
       </c>
       <c r="J60">
@@ -4649,7 +4736,7 @@
       <c r="H61" t="s">
         <v>63</v>
       </c>
-      <c r="I61">
+      <c r="I61" s="21">
         <v>6400</v>
       </c>
       <c r="J61">
@@ -4713,7 +4800,7 @@
       <c r="H62" t="s">
         <v>54</v>
       </c>
-      <c r="I62">
+      <c r="I62" s="21">
         <v>6295</v>
       </c>
       <c r="J62">
@@ -4777,7 +4864,7 @@
       <c r="H63" t="s">
         <v>66</v>
       </c>
-      <c r="I63">
+      <c r="I63" s="21">
         <v>6643</v>
       </c>
       <c r="J63">
@@ -4820,7 +4907,7 @@
       <c r="A64" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="I64" s="16">
+      <c r="I64" s="22">
         <v>6161.02294921875</v>
       </c>
       <c r="J64" s="16">
@@ -4855,7 +4942,7 @@
       <c r="B65" t="s">
         <v>20</v>
       </c>
-      <c r="I65">
+      <c r="I65" s="21">
         <v>6200</v>
       </c>
       <c r="J65">
@@ -4903,7 +4990,7 @@
       <c r="H66" t="s">
         <v>43</v>
       </c>
-      <c r="I66">
+      <c r="I66" s="21">
         <v>5990</v>
       </c>
       <c r="J66">
@@ -4967,7 +5054,7 @@
       <c r="H67" t="s">
         <v>56</v>
       </c>
-      <c r="I67">
+      <c r="I67" s="21">
         <v>6250</v>
       </c>
       <c r="J67">
@@ -5028,7 +5115,7 @@
       <c r="G68">
         <v>1872</v>
       </c>
-      <c r="I68">
+      <c r="I68" s="21">
         <v>6475</v>
       </c>
       <c r="J68">
@@ -5092,7 +5179,7 @@
       <c r="H69" t="s">
         <v>74</v>
       </c>
-      <c r="I69">
+      <c r="I69" s="21">
         <v>6050</v>
       </c>
       <c r="J69">
@@ -5156,7 +5243,7 @@
       <c r="H70" t="s">
         <v>118</v>
       </c>
-      <c r="I70">
+      <c r="I70" s="21">
         <v>9360</v>
       </c>
       <c r="J70">
@@ -5220,7 +5307,7 @@
       <c r="H71" t="s">
         <v>72</v>
       </c>
-      <c r="I71">
+      <c r="I71" s="21">
         <v>6432</v>
       </c>
       <c r="J71">
@@ -5282,7 +5369,7 @@
         <v>3353</v>
       </c>
       <c r="H72" s="6"/>
-      <c r="I72" s="6">
+      <c r="I72" s="24">
         <v>8000</v>
       </c>
       <c r="J72" s="6">
@@ -5349,7 +5436,7 @@
       <c r="H73" t="s">
         <v>41</v>
       </c>
-      <c r="I73">
+      <c r="I73" s="21">
         <v>7430</v>
       </c>
       <c r="J73">
@@ -5413,7 +5500,7 @@
       <c r="H74" t="s">
         <v>70</v>
       </c>
-      <c r="I74">
+      <c r="I74" s="21">
         <v>6180</v>
       </c>
       <c r="J74">
@@ -5477,7 +5564,7 @@
       <c r="H75" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="I75" s="6">
+      <c r="I75" s="24">
         <v>4792</v>
       </c>
       <c r="J75" s="6">
@@ -5541,7 +5628,7 @@
       <c r="G76">
         <v>1487</v>
       </c>
-      <c r="I76">
+      <c r="I76" s="21">
         <v>6400</v>
       </c>
       <c r="J76">
@@ -5605,7 +5692,7 @@
       <c r="H77" t="s">
         <v>91</v>
       </c>
-      <c r="I77">
+      <c r="I77" s="21">
         <v>5990</v>
       </c>
       <c r="J77">
@@ -5669,7 +5756,7 @@
       <c r="H78" t="s">
         <v>52</v>
       </c>
-      <c r="I78">
+      <c r="I78" s="21">
         <v>6329</v>
       </c>
       <c r="J78">
@@ -5733,7 +5820,7 @@
       <c r="H79" t="s">
         <v>127</v>
       </c>
-      <c r="I79">
+      <c r="I79" s="21">
         <v>6600</v>
       </c>
       <c r="J79">
@@ -5797,7 +5884,7 @@
       <c r="H80" t="s">
         <v>97</v>
       </c>
-      <c r="I80">
+      <c r="I80" s="21">
         <v>5600</v>
       </c>
       <c r="J80">
@@ -5836,7 +5923,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>132</v>
       </c>
@@ -5861,7 +5948,7 @@
       <c r="H81" t="s">
         <v>127</v>
       </c>
-      <c r="I81" s="15">
+      <c r="I81" s="26">
         <v>6480</v>
       </c>
       <c r="J81" s="15">
@@ -5900,7 +5987,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A82" s="12" t="s">
         <v>128</v>
       </c>
@@ -5925,7 +6012,7 @@
       <c r="H82" t="s">
         <v>54</v>
       </c>
-      <c r="I82" s="15">
+      <c r="I82" s="26">
         <v>6170</v>
       </c>
       <c r="J82" s="15">
@@ -5964,7 +6051,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A83" s="12" t="s">
         <v>133</v>
       </c>
@@ -5989,7 +6076,7 @@
       <c r="H83" t="s">
         <v>134</v>
       </c>
-      <c r="I83" s="15">
+      <c r="I83" s="26">
         <v>5830</v>
       </c>
       <c r="J83" s="15">
@@ -6028,7 +6115,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A84" s="12" t="s">
         <v>79</v>
       </c>
@@ -6053,7 +6140,7 @@
       <c r="H84" t="s">
         <v>54</v>
       </c>
-      <c r="I84" s="15">
+      <c r="I84" s="26">
         <v>6150</v>
       </c>
       <c r="J84" s="15">
@@ -6092,7 +6179,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A85" s="12" t="s">
         <v>107</v>
       </c>
@@ -6117,7 +6204,7 @@
       <c r="H85" t="s">
         <v>108</v>
       </c>
-      <c r="I85" s="17">
+      <c r="I85" s="27">
         <v>6429</v>
       </c>
       <c r="J85" s="17">
@@ -6156,8 +6243,170 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A86" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="I86" s="26">
+        <v>3460</v>
+      </c>
+      <c r="J86" s="15">
+        <v>0.54700000000000004</v>
+      </c>
+      <c r="K86">
+        <v>0.54300000000000004</v>
+      </c>
+      <c r="L86">
+        <v>0</v>
+      </c>
+      <c r="M86">
+        <v>4.6963999999999997</v>
+      </c>
+      <c r="N86">
+        <v>303.19871318011002</v>
+      </c>
+      <c r="O86">
+        <v>-0.37849292589</v>
+      </c>
+      <c r="P86">
+        <v>312.65899999999999</v>
+      </c>
       <c r="R86"/>
+      <c r="V86">
+        <v>10.968999999999999</v>
+      </c>
+      <c r="W86">
+        <v>11.454000000000001</v>
+      </c>
+      <c r="X86" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y86" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="87" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A87" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="I87" s="26">
+        <v>3496</v>
+      </c>
+      <c r="J87" s="15">
+        <v>83.710999999999999</v>
+      </c>
+      <c r="K87">
+        <v>0</v>
+      </c>
+      <c r="L87">
+        <v>0</v>
+      </c>
+      <c r="M87">
+        <v>0</v>
+      </c>
+      <c r="N87">
+        <v>293.64838257128002</v>
+      </c>
+      <c r="O87">
+        <v>-12.35499539692</v>
+      </c>
+      <c r="P87">
+        <v>1655.31</v>
+      </c>
+      <c r="V87">
+        <v>10.977</v>
+      </c>
+      <c r="W87">
+        <v>12.571999999999999</v>
+      </c>
+      <c r="X87" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y87" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="88" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>152</v>
+      </c>
+      <c r="I88" s="21">
+        <v>5827</v>
+      </c>
+      <c r="J88">
+        <v>6.9720000000000004</v>
+      </c>
+      <c r="K88">
+        <v>0</v>
+      </c>
+      <c r="L88">
+        <v>0</v>
+      </c>
+      <c r="M88">
+        <v>0</v>
+      </c>
+      <c r="N88">
+        <v>12.295169568029999</v>
+      </c>
+      <c r="O88">
+        <v>-40.067873380309997</v>
+      </c>
+      <c r="P88">
+        <v>1154.6099999999999</v>
+      </c>
+      <c r="V88">
+        <v>10.988</v>
+      </c>
+      <c r="W88">
+        <v>11.585000000000001</v>
+      </c>
+      <c r="X88" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y88" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="89" spans="1:25" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>153</v>
+      </c>
+      <c r="I89" s="21">
+        <v>5798</v>
+      </c>
+      <c r="J89">
+        <v>1.288</v>
+      </c>
+      <c r="K89">
+        <v>1.04</v>
+      </c>
+      <c r="L89">
+        <v>0</v>
+      </c>
+      <c r="M89">
+        <v>4.2351999999999999</v>
+      </c>
+      <c r="N89">
+        <v>78.92072949976</v>
+      </c>
+      <c r="O89">
+        <v>-61.051005597089997</v>
+      </c>
+      <c r="P89">
+        <v>216.126</v>
+      </c>
+      <c r="V89">
+        <v>11.000999999999999</v>
+      </c>
+      <c r="W89">
+        <v>11.773999999999999</v>
+      </c>
+      <c r="X89" t="s">
+        <v>149</v>
+      </c>
+      <c r="Y89" t="s">
+        <v>137</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U79" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
renamed 1 to 01 percent. because we changed psf
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0F22DF-0304-404A-9524-A0448C59AB02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9B7E04-4FBA-F649-BE77-51F16EC5FCFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="174">
   <si>
     <t>#pl_name</t>
   </si>
@@ -531,6 +531,33 @@
   </si>
   <si>
     <t>4037578191010248064 b</t>
+  </si>
+  <si>
+    <t>VMAG11 b</t>
+  </si>
+  <si>
+    <t>VMAG12 b</t>
+  </si>
+  <si>
+    <t>VMAG13 b</t>
+  </si>
+  <si>
+    <t>VMAG14 b</t>
+  </si>
+  <si>
+    <t>VMAG15 b</t>
+  </si>
+  <si>
+    <t>VMAG16 b</t>
+  </si>
+  <si>
+    <t>VMAG17 b</t>
+  </si>
+  <si>
+    <t>VMAG18 b</t>
+  </si>
+  <si>
+    <t>VMAG19 b</t>
   </si>
 </sst>
 </file>
@@ -936,15 +963,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BB101"/>
+  <dimension ref="A1:BB110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="12.1640625" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5" hidden="1" customWidth="1"/>
-    <col min="5" max="6" width="11.1640625" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="8.5" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.1640625" customWidth="1"/>
+    <col min="4" max="4" width="12.5" customWidth="1"/>
+    <col min="5" max="6" width="11.1640625" customWidth="1"/>
+    <col min="7" max="7" width="8.5" customWidth="1"/>
     <col min="8" max="8" width="12.5" customWidth="1"/>
     <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.1640625" bestFit="1" customWidth="1"/>
@@ -6768,6 +6795,258 @@
         <v>9.2583198549999999</v>
       </c>
     </row>
+    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
+      <c r="I102" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J102">
+        <v>0.4</v>
+      </c>
+      <c r="K102">
+        <v>0.4</v>
+      </c>
+      <c r="N102">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O102">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P102">
+        <v>11</v>
+      </c>
+      <c r="Q102">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B103" s="1"/>
+      <c r="C103" s="1"/>
+      <c r="D103" s="1"/>
+      <c r="E103" s="1"/>
+      <c r="F103" s="1"/>
+      <c r="G103" s="1"/>
+      <c r="I103" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J103">
+        <v>0.4</v>
+      </c>
+      <c r="K103">
+        <v>0.4</v>
+      </c>
+      <c r="N103">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O103">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P103">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="Q103">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B104" s="1"/>
+      <c r="C104" s="1"/>
+      <c r="D104" s="1"/>
+      <c r="E104" s="1"/>
+      <c r="F104" s="1"/>
+      <c r="G104" s="1"/>
+      <c r="I104" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J104">
+        <v>0.4</v>
+      </c>
+      <c r="K104">
+        <v>0.4</v>
+      </c>
+      <c r="N104">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O104">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P104">
+        <v>27.5</v>
+      </c>
+      <c r="Q104">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="I105" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J105">
+        <v>0.4</v>
+      </c>
+      <c r="K105">
+        <v>0.4</v>
+      </c>
+      <c r="N105">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O105">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P105">
+        <v>43.7</v>
+      </c>
+      <c r="Q105">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="I106" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J106">
+        <v>0.4</v>
+      </c>
+      <c r="K106">
+        <v>0.4</v>
+      </c>
+      <c r="N106">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O106">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P106">
+        <v>69.2</v>
+      </c>
+      <c r="Q106">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="I107" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J107">
+        <v>0.4</v>
+      </c>
+      <c r="K107">
+        <v>0.4</v>
+      </c>
+      <c r="N107">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O107">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P107">
+        <v>109.6</v>
+      </c>
+      <c r="Q107">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I108" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J108">
+        <v>0.4</v>
+      </c>
+      <c r="K108">
+        <v>0.4</v>
+      </c>
+      <c r="N108">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O108">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P108">
+        <v>173.8</v>
+      </c>
+      <c r="Q108">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="I109" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J109">
+        <v>0.4</v>
+      </c>
+      <c r="K109">
+        <v>0.4</v>
+      </c>
+      <c r="N109">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O109">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P109">
+        <v>275.39999999999998</v>
+      </c>
+      <c r="Q109">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="I110" s="1">
+        <v>3500</v>
+      </c>
+      <c r="J110">
+        <v>0.4</v>
+      </c>
+      <c r="K110">
+        <v>0.4</v>
+      </c>
+      <c r="N110">
+        <v>346.62201299999998</v>
+      </c>
+      <c r="O110">
+        <v>-5.0412739999999996</v>
+      </c>
+      <c r="P110">
+        <v>436.5</v>
+      </c>
+      <c r="Q110">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:W100" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R77">

</xml_diff>

<commit_message>
added shared common function for background star calculations
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F9B7E04-4FBA-F649-BE77-51F16EC5FCFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6B6557-630B-6746-BD1C-21D76F1AD0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5214,36 +5214,6 @@
       <c r="G75">
         <v>1439</v>
       </c>
-      <c r="I75">
-        <v>6110</v>
-      </c>
-      <c r="J75">
-        <v>1.6479999999999999</v>
-      </c>
-      <c r="K75">
-        <v>1.2909999999999999</v>
-      </c>
-      <c r="L75">
-        <v>0.124</v>
-      </c>
-      <c r="M75">
-        <v>4.1180000000000003</v>
-      </c>
-      <c r="N75">
-        <v>51.657269100000001</v>
-      </c>
-      <c r="O75">
-        <v>40.817270399999998</v>
-      </c>
-      <c r="P75">
-        <v>179.14699999999999</v>
-      </c>
-      <c r="Q75">
-        <v>9.9130000000000003</v>
-      </c>
-      <c r="R75">
-        <v>9.7295700000000007</v>
-      </c>
       <c r="S75">
         <f t="shared" si="2"/>
         <v>487.59044264912109</v>

</xml_diff>

<commit_message>
store parallax all the time when requesting gaia to make distance fallback
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6B6557-630B-6746-BD1C-21D76F1AD0F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC1F409-F173-C545-82B1-341278B72042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Targets_V10p1!$A$1:$W$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Targets_V10p1!$A$1:$W$110</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="173">
   <si>
     <t>#pl_name</t>
   </si>
@@ -459,9 +459,6 @@
   </si>
   <si>
     <t>HAT-P-7 b</t>
-  </si>
-  <si>
-    <t>B9.5-A0</t>
   </si>
   <si>
     <t>B_MAG</t>
@@ -564,10 +561,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="0.000000_ "/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -594,6 +592,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -658,12 +663,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -688,8 +694,15 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -963,6 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:BB110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -982,9 +996,9 @@
     <col min="16" max="16" width="9.1640625" customWidth="1"/>
     <col min="17" max="17" width="12.1640625" customWidth="1"/>
     <col min="18" max="18" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.1640625" hidden="1" customWidth="1"/>
-    <col min="20" max="20" width="7" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="13.33203125" hidden="1" customWidth="1"/>
+    <col min="19" max="19" width="16.1640625" customWidth="1"/>
+    <col min="20" max="20" width="7" customWidth="1"/>
+    <col min="21" max="21" width="13.33203125" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="9"/>
@@ -1066,15 +1080,15 @@
         <v>136</v>
       </c>
       <c r="V1" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="W1" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="W1" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="2" spans="1:54" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I2">
         <v>3501</v>
@@ -1107,15 +1121,15 @@
         <v>12.885999999999999</v>
       </c>
       <c r="W2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AY2" s="3"/>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
     </row>
-    <row r="3" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I3">
         <v>3496</v>
@@ -1148,15 +1162,15 @@
         <v>12.571999999999999</v>
       </c>
       <c r="W3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="AY3" s="3"/>
       <c r="BA3" s="3"/>
       <c r="BB3" s="3"/>
     </row>
-    <row r="4" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I4">
         <v>3460</v>
@@ -1189,15 +1203,15 @@
         <v>11.454000000000001</v>
       </c>
       <c r="W4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AY4" s="3"/>
       <c r="BA4" s="3"/>
       <c r="BB4" s="3"/>
     </row>
-    <row r="5" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I5">
         <v>5804</v>
@@ -1230,15 +1244,15 @@
         <v>16.86</v>
       </c>
       <c r="W5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AY5" s="3"/>
       <c r="BA5" s="3"/>
       <c r="BB5" s="3"/>
     </row>
-    <row r="6" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I6">
         <v>5800</v>
@@ -1271,15 +1285,15 @@
         <v>17.364000000000001</v>
       </c>
       <c r="W6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="AY6" s="3"/>
       <c r="BA6" s="3"/>
       <c r="BB6" s="3"/>
     </row>
-    <row r="7" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I7">
         <v>5799</v>
@@ -1312,12 +1326,12 @@
         <v>12.47</v>
       </c>
       <c r="W7" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="8" spans="1:54" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I8">
         <v>5800.4</v>
@@ -1350,12 +1364,12 @@
         <v>13.638999999999999</v>
       </c>
       <c r="W8" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="9" spans="1:54" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I9">
         <v>5813</v>
@@ -1388,12 +1402,12 @@
         <v>15.66</v>
       </c>
       <c r="W9" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10" spans="1:54" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I10">
         <v>5820</v>
@@ -1426,12 +1440,12 @@
         <v>15.702999999999999</v>
       </c>
       <c r="W10" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="11" spans="1:54" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="11" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I11">
         <v>5824</v>
@@ -1464,12 +1478,12 @@
         <v>15.048999999999999</v>
       </c>
       <c r="W11" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="12" spans="1:54" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="12" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I12">
         <v>5816</v>
@@ -1502,12 +1516,12 @@
         <v>17.585999999999999</v>
       </c>
       <c r="W12" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="13" spans="1:54" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I13">
         <v>5792</v>
@@ -1540,9 +1554,9 @@
         <v>18.082999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:54" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I14">
         <v>5775</v>
@@ -1575,12 +1589,12 @@
         <v>14.082000000000001</v>
       </c>
       <c r="W14" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="15" spans="1:54" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="15" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I15">
         <v>5800</v>
@@ -1613,12 +1627,12 @@
         <v>14.913</v>
       </c>
       <c r="W15" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16" spans="1:54" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I16">
         <v>5806</v>
@@ -1651,12 +1665,12 @@
         <v>12.507</v>
       </c>
       <c r="W16" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I17">
         <v>5815.4</v>
@@ -1689,12 +1703,12 @@
         <v>11.56</v>
       </c>
       <c r="W17" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I18">
         <v>5812</v>
@@ -1727,10 +1741,10 @@
         <v>11.662000000000001</v>
       </c>
       <c r="W18" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -1794,7 +1808,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>124</v>
       </c>
@@ -1858,7 +1872,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -1922,7 +1936,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -1986,7 +2000,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>139</v>
       </c>
@@ -2015,7 +2029,7 @@
         <v>11.12930202484131</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>88</v>
       </c>
@@ -2076,7 +2090,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>95</v>
       </c>
@@ -2137,7 +2151,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>140</v>
       </c>
@@ -2160,7 +2174,7 @@
         <v>10.36768245697021</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -2221,7 +2235,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -2285,7 +2299,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -2349,7 +2363,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -2413,7 +2427,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>59</v>
       </c>
@@ -2477,7 +2491,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -2541,7 +2555,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>50</v>
       </c>
@@ -2602,7 +2616,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>25</v>
       </c>
@@ -2666,7 +2680,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -2730,7 +2744,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -2816,49 +2830,11 @@
       <c r="G37">
         <v>2061</v>
       </c>
-      <c r="I37">
-        <v>6801</v>
-      </c>
-      <c r="J37">
-        <v>1.56</v>
-      </c>
-      <c r="K37">
-        <v>1.43</v>
-      </c>
-      <c r="L37">
-        <v>0.02</v>
-      </c>
-      <c r="M37">
-        <v>4.21</v>
-      </c>
-      <c r="N37">
-        <v>7.3289156000000002</v>
-      </c>
-      <c r="O37">
-        <v>-76.304032000000007</v>
-      </c>
-      <c r="P37">
-        <v>196.852</v>
-      </c>
-      <c r="Q37">
-        <v>9.5950000000000006</v>
-      </c>
-      <c r="R37">
-        <v>9.5202500000000008</v>
-      </c>
-      <c r="S37">
-        <f t="shared" si="0"/>
-        <v>934.76971602454307</v>
-      </c>
-      <c r="T37">
-        <f t="shared" si="1"/>
-        <v>-7</v>
-      </c>
       <c r="U37" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>53</v>
       </c>
@@ -2922,7 +2898,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -2986,7 +2962,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -3050,7 +3026,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -3111,7 +3087,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>36</v>
       </c>
@@ -3175,7 +3151,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>67</v>
       </c>
@@ -3239,7 +3215,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>109</v>
       </c>
@@ -3303,7 +3279,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>57</v>
       </c>
@@ -3367,7 +3343,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>23</v>
       </c>
@@ -3431,7 +3407,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -3495,7 +3471,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>103</v>
       </c>
@@ -3556,7 +3532,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>123</v>
       </c>
@@ -3620,7 +3596,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -3706,48 +3682,11 @@
       <c r="G51">
         <v>4050</v>
       </c>
-      <c r="H51" t="s">
-        <v>141</v>
-      </c>
-      <c r="I51">
-        <v>10170.1</v>
-      </c>
-      <c r="J51">
-        <v>2.3620000000000001</v>
-      </c>
-      <c r="K51">
-        <v>2.52</v>
-      </c>
-      <c r="L51">
-        <v>-0.03</v>
-      </c>
-      <c r="M51">
-        <v>4.093</v>
-      </c>
-      <c r="N51">
-        <v>307.85989979999999</v>
-      </c>
-      <c r="O51">
-        <v>39.9389161</v>
-      </c>
-      <c r="P51">
-        <v>204.45500000000001</v>
-      </c>
-      <c r="Q51">
-        <v>7.55</v>
-      </c>
-      <c r="R51">
-        <v>7.5767499999999997</v>
-      </c>
-      <c r="S51">
-        <f t="shared" si="0"/>
-        <v>1286.8653667451285</v>
-      </c>
       <c r="U51" s="1" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -3808,7 +3747,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>98</v>
       </c>
@@ -3872,7 +3811,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>48</v>
       </c>
@@ -3936,7 +3875,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>46</v>
       </c>
@@ -4067,7 +4006,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>84</v>
       </c>
@@ -4131,7 +4070,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>83</v>
       </c>
@@ -4192,7 +4131,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>77</v>
       </c>
@@ -4253,7 +4192,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>69</v>
       </c>
@@ -4317,7 +4256,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>34</v>
       </c>
@@ -4381,7 +4320,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>60</v>
       </c>
@@ -4445,7 +4384,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>87</v>
       </c>
@@ -4509,7 +4448,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>102</v>
       </c>
@@ -4570,7 +4509,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>111</v>
       </c>
@@ -4631,7 +4570,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>64</v>
       </c>
@@ -4692,7 +4631,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>85</v>
       </c>
@@ -4753,7 +4692,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -4814,7 +4753,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>115</v>
       </c>
@@ -4878,7 +4817,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>121</v>
       </c>
@@ -4939,7 +4878,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>68</v>
       </c>
@@ -5003,7 +4942,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>119</v>
       </c>
@@ -5067,7 +5006,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>92</v>
       </c>
@@ -5128,7 +5067,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>129</v>
       </c>
@@ -5192,7 +5131,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>114</v>
       </c>
@@ -5214,16 +5153,17 @@
       <c r="G75">
         <v>1439</v>
       </c>
-      <c r="S75">
-        <f t="shared" si="2"/>
-        <v>487.59044264912109</v>
-      </c>
-      <c r="T75">
-        <f t="shared" si="3"/>
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="N75" s="8">
+        <v>51.657269100000001</v>
+      </c>
+      <c r="O75" s="9">
+        <v>40.817270399999998</v>
+      </c>
+      <c r="U75" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>62</v>
       </c>
@@ -5287,7 +5227,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>105</v>
       </c>
@@ -5351,7 +5291,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>65</v>
       </c>
@@ -5415,7 +5355,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>138</v>
       </c>
@@ -5445,7 +5385,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>131</v>
       </c>
@@ -5509,7 +5449,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>122</v>
       </c>
@@ -5573,7 +5513,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>89</v>
       </c>
@@ -5634,7 +5574,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>73</v>
       </c>
@@ -5698,7 +5638,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>117</v>
       </c>
@@ -5762,7 +5702,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>71</v>
       </c>
@@ -5890,7 +5830,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>40</v>
       </c>
@@ -5954,7 +5894,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>76</v>
       </c>
@@ -6085,7 +6025,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>81</v>
       </c>
@@ -6146,7 +6086,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>90</v>
       </c>
@@ -6210,7 +6150,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>82</v>
       </c>
@@ -6274,9 +6214,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="I93" s="1">
         <v>3472</v>
@@ -6297,7 +6237,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>126</v>
       </c>
@@ -6361,7 +6301,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>96</v>
       </c>
@@ -6425,7 +6365,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>132</v>
       </c>
@@ -6489,7 +6429,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>128</v>
       </c>
@@ -6553,7 +6493,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>133</v>
       </c>
@@ -6617,7 +6557,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>79</v>
       </c>
@@ -6681,7 +6621,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>107</v>
       </c>
@@ -6745,9 +6685,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="101" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I101">
         <v>7065.3916019999997</v>
@@ -6765,9 +6705,9 @@
         <v>9.2583198549999999</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -6797,9 +6737,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -6829,9 +6769,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -6861,9 +6801,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I105" s="1">
         <v>3500</v>
@@ -6887,9 +6827,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I106" s="1">
         <v>3500</v>
@@ -6913,9 +6853,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I107" s="1">
         <v>3500</v>
@@ -6939,9 +6879,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I108" s="1">
         <v>3500</v>
@@ -6965,9 +6905,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I109" s="1">
         <v>3500</v>
@@ -6991,9 +6931,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="I110" s="1">
         <v>3500</v>
@@ -7018,7 +6958,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W100" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:W110" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="20">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R77">
     <sortCondition ref="Q2"/>
   </sortState>

</xml_diff>

<commit_message>
added new background star csvs
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC1F409-F173-C545-82B1-341278B72042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493AB0B3-DF4C-8643-BE7F-6065918041ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Targets_V10p1!$A$1:$W$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Targets_V10p1!$A$1:$W$100</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="174">
   <si>
     <t>#pl_name</t>
   </si>
@@ -365,9 +365,6 @@
     <t>F5V</t>
   </si>
   <si>
-    <t>KELT-19 A b</t>
-  </si>
-  <si>
     <t>A8 V</t>
   </si>
   <si>
@@ -380,9 +377,6 @@
     <t>K</t>
   </si>
   <si>
-    <t>TOI-6038 A b</t>
-  </si>
-  <si>
     <t>TOI-421 c</t>
   </si>
   <si>
@@ -461,6 +455,9 @@
     <t>HAT-P-7 b</t>
   </si>
   <si>
+    <t>B9.5-A0</t>
+  </si>
+  <si>
     <t>B_MAG</t>
   </si>
   <si>
@@ -555,17 +552,22 @@
   </si>
   <si>
     <t>VMAG19 b</t>
+  </si>
+  <si>
+    <t>TOI-6038 b</t>
+  </si>
+  <si>
+    <t>KELT-19 b</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000_ "/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -592,13 +594,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -663,13 +658,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -694,15 +688,8 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -976,7 +963,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:BB110"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
@@ -996,9 +982,9 @@
     <col min="16" max="16" width="9.1640625" customWidth="1"/>
     <col min="17" max="17" width="12.1640625" customWidth="1"/>
     <col min="18" max="18" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.1640625" customWidth="1"/>
-    <col min="20" max="20" width="7" customWidth="1"/>
-    <col min="21" max="21" width="13.33203125" customWidth="1"/>
+    <col min="19" max="19" width="16.1640625" hidden="1" customWidth="1"/>
+    <col min="20" max="20" width="7" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="13.33203125" hidden="1" customWidth="1"/>
     <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="9.83203125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="9"/>
@@ -1074,21 +1060,21 @@
         <v>18</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="V1" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="W1" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="W1" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="2" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I2">
         <v>3501</v>
@@ -1121,15 +1107,15 @@
         <v>12.885999999999999</v>
       </c>
       <c r="W2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AY2" s="3"/>
       <c r="BA2" s="3"/>
       <c r="BB2" s="3"/>
     </row>
-    <row r="3" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I3">
         <v>3496</v>
@@ -1162,15 +1148,15 @@
         <v>12.571999999999999</v>
       </c>
       <c r="W3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="AY3" s="3"/>
       <c r="BA3" s="3"/>
       <c r="BB3" s="3"/>
     </row>
-    <row r="4" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I4">
         <v>3460</v>
@@ -1203,15 +1189,15 @@
         <v>11.454000000000001</v>
       </c>
       <c r="W4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AY4" s="3"/>
       <c r="BA4" s="3"/>
       <c r="BB4" s="3"/>
     </row>
-    <row r="5" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I5">
         <v>5804</v>
@@ -1244,15 +1230,15 @@
         <v>16.86</v>
       </c>
       <c r="W5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AY5" s="3"/>
       <c r="BA5" s="3"/>
       <c r="BB5" s="3"/>
     </row>
-    <row r="6" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I6">
         <v>5800</v>
@@ -1285,15 +1271,15 @@
         <v>17.364000000000001</v>
       </c>
       <c r="W6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="AY6" s="3"/>
       <c r="BA6" s="3"/>
       <c r="BB6" s="3"/>
     </row>
-    <row r="7" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I7">
         <v>5799</v>
@@ -1326,12 +1312,12 @@
         <v>12.47</v>
       </c>
       <c r="W7" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="8" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="8" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I8">
         <v>5800.4</v>
@@ -1364,12 +1350,12 @@
         <v>13.638999999999999</v>
       </c>
       <c r="W8" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="9" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I9">
         <v>5813</v>
@@ -1402,12 +1388,12 @@
         <v>15.66</v>
       </c>
       <c r="W9" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="10" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="10" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I10">
         <v>5820</v>
@@ -1440,12 +1426,12 @@
         <v>15.702999999999999</v>
       </c>
       <c r="W10" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="11" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I11">
         <v>5824</v>
@@ -1478,12 +1464,12 @@
         <v>15.048999999999999</v>
       </c>
       <c r="W11" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="12" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="12" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="I12">
         <v>5816</v>
@@ -1516,12 +1502,12 @@
         <v>17.585999999999999</v>
       </c>
       <c r="W12" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="13" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="13" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I13">
         <v>5792</v>
@@ -1554,9 +1540,9 @@
         <v>18.082999999999998</v>
       </c>
     </row>
-    <row r="14" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I14">
         <v>5775</v>
@@ -1589,12 +1575,12 @@
         <v>14.082000000000001</v>
       </c>
       <c r="W14" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="15" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="15" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I15">
         <v>5800</v>
@@ -1627,12 +1613,12 @@
         <v>14.913</v>
       </c>
       <c r="W15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="16" spans="1:54" hidden="1" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I16">
         <v>5806</v>
@@ -1665,12 +1651,12 @@
         <v>12.507</v>
       </c>
       <c r="W16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I17">
         <v>5815.4</v>
@@ -1703,12 +1689,12 @@
         <v>11.56</v>
       </c>
       <c r="W17" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I18">
         <v>5812</v>
@@ -1741,10 +1727,10 @@
         <v>11.662000000000001</v>
       </c>
       <c r="W18" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>106</v>
       </c>
@@ -1808,9 +1794,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="20" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
@@ -1831,7 +1817,7 @@
         <v>1624</v>
       </c>
       <c r="H20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I20">
         <v>6600</v>
@@ -1872,7 +1858,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="21" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>58</v>
       </c>
@@ -1936,7 +1922,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="22" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -2000,9 +1986,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="23" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I23">
         <v>6245.11328125</v>
@@ -2029,7 +2015,7 @@
         <v>11.12930202484131</v>
       </c>
     </row>
-    <row r="24" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>88</v>
       </c>
@@ -2090,7 +2076,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="25" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>95</v>
       </c>
@@ -2151,9 +2137,9 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="26" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I26">
         <v>6424.27685546875</v>
@@ -2174,7 +2160,7 @@
         <v>10.36768245697021</v>
       </c>
     </row>
-    <row r="27" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -2235,7 +2221,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="28" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -2299,7 +2285,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="29" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -2363,7 +2349,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>42</v>
       </c>
@@ -2427,7 +2413,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="31" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>59</v>
       </c>
@@ -2491,7 +2477,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="32" spans="1:23" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -2555,7 +2541,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="33" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>50</v>
       </c>
@@ -2616,7 +2602,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="34" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>25</v>
       </c>
@@ -2680,7 +2666,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="35" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>101</v>
       </c>
@@ -2744,7 +2730,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="36" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -2830,11 +2816,49 @@
       <c r="G37">
         <v>2061</v>
       </c>
+      <c r="I37">
+        <v>6801</v>
+      </c>
+      <c r="J37">
+        <v>1.56</v>
+      </c>
+      <c r="K37">
+        <v>1.43</v>
+      </c>
+      <c r="L37">
+        <v>0.02</v>
+      </c>
+      <c r="M37">
+        <v>4.21</v>
+      </c>
+      <c r="N37">
+        <v>7.3289156000000002</v>
+      </c>
+      <c r="O37">
+        <v>-76.304032000000007</v>
+      </c>
+      <c r="P37">
+        <v>196.852</v>
+      </c>
+      <c r="Q37">
+        <v>9.5950000000000006</v>
+      </c>
+      <c r="R37">
+        <v>9.5202500000000008</v>
+      </c>
+      <c r="S37">
+        <f t="shared" si="0"/>
+        <v>934.76971602454307</v>
+      </c>
+      <c r="T37">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
       <c r="U37" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="38" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>53</v>
       </c>
@@ -2898,7 +2922,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="39" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>32</v>
       </c>
@@ -2962,7 +2986,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="40" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>75</v>
       </c>
@@ -3026,7 +3050,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="41" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -3087,7 +3111,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="42" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>36</v>
       </c>
@@ -3151,7 +3175,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="43" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>67</v>
       </c>
@@ -3215,9 +3239,9 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="44" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
-        <v>109</v>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>173</v>
       </c>
       <c r="B44" t="s">
         <v>20</v>
@@ -3238,7 +3262,7 @@
         <v>1935</v>
       </c>
       <c r="H44" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="I44">
         <v>7500</v>
@@ -3279,7 +3303,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="45" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>57</v>
       </c>
@@ -3343,7 +3367,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="46" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>23</v>
       </c>
@@ -3407,7 +3431,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="47" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -3471,7 +3495,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="48" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>103</v>
       </c>
@@ -3532,9 +3556,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="49" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B49" t="s">
         <v>20</v>
@@ -3596,7 +3620,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="50" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -3682,11 +3706,48 @@
       <c r="G51">
         <v>4050</v>
       </c>
+      <c r="H51" t="s">
+        <v>139</v>
+      </c>
+      <c r="I51">
+        <v>10170.1</v>
+      </c>
+      <c r="J51">
+        <v>2.3620000000000001</v>
+      </c>
+      <c r="K51">
+        <v>2.52</v>
+      </c>
+      <c r="L51">
+        <v>-0.03</v>
+      </c>
+      <c r="M51">
+        <v>4.093</v>
+      </c>
+      <c r="N51">
+        <v>307.85989979999999</v>
+      </c>
+      <c r="O51">
+        <v>39.9389161</v>
+      </c>
+      <c r="P51">
+        <v>204.45500000000001</v>
+      </c>
+      <c r="Q51">
+        <v>7.55</v>
+      </c>
+      <c r="R51">
+        <v>7.5767499999999997</v>
+      </c>
+      <c r="S51">
+        <f t="shared" si="0"/>
+        <v>1286.8653667451285</v>
+      </c>
       <c r="U51" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -3747,7 +3808,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="53" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>98</v>
       </c>
@@ -3811,7 +3872,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="54" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>48</v>
       </c>
@@ -3875,7 +3936,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="55" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>46</v>
       </c>
@@ -4003,10 +4064,10 @@
         <v>-5</v>
       </c>
       <c r="U56" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="57" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>84</v>
       </c>
@@ -4070,7 +4131,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="58" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>83</v>
       </c>
@@ -4131,7 +4192,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="59" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>77</v>
       </c>
@@ -4192,7 +4253,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="60" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>69</v>
       </c>
@@ -4256,7 +4317,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="61" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>34</v>
       </c>
@@ -4320,7 +4381,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="62" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>60</v>
       </c>
@@ -4384,7 +4445,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="63" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>87</v>
       </c>
@@ -4448,7 +4509,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="64" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>102</v>
       </c>
@@ -4509,9 +4570,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="65" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B65" t="s">
         <v>20</v>
@@ -4570,7 +4631,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="66" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>64</v>
       </c>
@@ -4631,7 +4692,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="67" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>85</v>
       </c>
@@ -4692,7 +4753,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="68" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -4753,9 +4814,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="69" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B69" t="s">
         <v>20</v>
@@ -4776,7 +4837,7 @@
         <v>635</v>
       </c>
       <c r="H69" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I69">
         <v>5291</v>
@@ -4817,9 +4878,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="70" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B70" t="s">
         <v>20</v>
@@ -4878,7 +4939,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="71" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>68</v>
       </c>
@@ -4942,9 +5003,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="72" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B72" t="s">
         <v>20</v>
@@ -4965,7 +5026,7 @@
         <v>1370</v>
       </c>
       <c r="H72" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I72">
         <v>5735</v>
@@ -5006,7 +5067,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="73" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>92</v>
       </c>
@@ -5067,9 +5128,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="74" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B74" t="s">
         <v>20</v>
@@ -5090,7 +5151,7 @@
         <v>947</v>
       </c>
       <c r="H74" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I74">
         <v>6000</v>
@@ -5131,9 +5192,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
-        <v>114</v>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
+        <v>172</v>
       </c>
       <c r="B75" t="s">
         <v>20</v>
@@ -5153,17 +5214,46 @@
       <c r="G75">
         <v>1439</v>
       </c>
-      <c r="N75" s="8">
+      <c r="I75">
+        <v>6110</v>
+      </c>
+      <c r="J75">
+        <v>1.6479999999999999</v>
+      </c>
+      <c r="K75">
+        <v>1.2909999999999999</v>
+      </c>
+      <c r="L75">
+        <v>0.124</v>
+      </c>
+      <c r="M75">
+        <v>4.1180000000000003</v>
+      </c>
+      <c r="N75">
         <v>51.657269100000001</v>
       </c>
-      <c r="O75" s="9">
+      <c r="O75">
         <v>40.817270399999998</v>
       </c>
-      <c r="U75" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="76" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+      <c r="P75">
+        <v>179.14699999999999</v>
+      </c>
+      <c r="Q75">
+        <v>9.9130000000000003</v>
+      </c>
+      <c r="R75">
+        <v>9.7295700000000007</v>
+      </c>
+      <c r="S75">
+        <f t="shared" si="2"/>
+        <v>487.59044264912109</v>
+      </c>
+      <c r="T75">
+        <f t="shared" si="3"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>62</v>
       </c>
@@ -5227,7 +5317,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="77" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>105</v>
       </c>
@@ -5291,7 +5381,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="78" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>65</v>
       </c>
@@ -5355,9 +5445,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="79" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B79" t="s">
         <v>20</v>
@@ -5385,9 +5475,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="80" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B80" t="s">
         <v>20</v>
@@ -5449,9 +5539,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="81" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B81" t="s">
         <v>20</v>
@@ -5513,7 +5603,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="82" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>89</v>
       </c>
@@ -5574,7 +5664,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="83" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>73</v>
       </c>
@@ -5638,9 +5728,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="84" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B84" t="s">
         <v>20</v>
@@ -5661,7 +5751,7 @@
         <v>2470</v>
       </c>
       <c r="H84" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="I84">
         <v>9360</v>
@@ -5702,7 +5792,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="85" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>71</v>
       </c>
@@ -5827,10 +5917,10 @@
         <v>-7</v>
       </c>
       <c r="U86" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="87" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>40</v>
       </c>
@@ -5894,7 +5984,7 @@
         <v>-7</v>
       </c>
     </row>
-    <row r="88" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>76</v>
       </c>
@@ -5960,7 +6050,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B89" t="s">
         <v>20</v>
@@ -5981,7 +6071,7 @@
         <v>971</v>
       </c>
       <c r="H89" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I89">
         <v>4792</v>
@@ -6022,10 +6112,10 @@
         <v>-5</v>
       </c>
       <c r="U89" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="90" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="90" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>81</v>
       </c>
@@ -6086,7 +6176,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="91" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>90</v>
       </c>
@@ -6150,7 +6240,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="92" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>82</v>
       </c>
@@ -6214,9 +6304,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="93" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A93" s="7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I93" s="1">
         <v>3472</v>
@@ -6237,9 +6327,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B94" t="s">
         <v>20</v>
@@ -6260,7 +6350,7 @@
         <v>1716.2</v>
       </c>
       <c r="H94" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I94">
         <v>6600</v>
@@ -6301,7 +6391,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="95" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>96</v>
       </c>
@@ -6365,9 +6455,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="96" spans="1:21" hidden="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B96" t="s">
         <v>20</v>
@@ -6388,7 +6478,7 @@
         <v>2190</v>
       </c>
       <c r="H96" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="I96">
         <v>6480</v>
@@ -6429,9 +6519,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="97" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B97" t="s">
         <v>20</v>
@@ -6493,9 +6583,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="98" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B98" t="s">
         <v>20</v>
@@ -6516,7 +6606,7 @@
         <v>1570</v>
       </c>
       <c r="H98" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I98">
         <v>5830</v>
@@ -6557,7 +6647,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="99" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>79</v>
       </c>
@@ -6621,7 +6711,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="100" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>107</v>
       </c>
@@ -6685,9 +6775,9 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="101" spans="1:20" ht="16" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I101">
         <v>7065.3916019999997</v>
@@ -6705,9 +6795,9 @@
         <v>9.2583198549999999</v>
       </c>
     </row>
-    <row r="102" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B102" s="1"/>
       <c r="C102" s="1"/>
@@ -6737,9 +6827,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B103" s="1"/>
       <c r="C103" s="1"/>
@@ -6769,9 +6859,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B104" s="1"/>
       <c r="C104" s="1"/>
@@ -6801,9 +6891,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I105" s="1">
         <v>3500</v>
@@ -6827,9 +6917,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="106" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="I106" s="1">
         <v>3500</v>
@@ -6853,9 +6943,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="107" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="I107" s="1">
         <v>3500</v>
@@ -6879,9 +6969,9 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="I108" s="1">
         <v>3500</v>
@@ -6905,9 +6995,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="I109" s="1">
         <v>3500</v>
@@ -6931,9 +7021,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="110" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I110" s="1">
         <v>3500</v>
@@ -6958,13 +7048,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W110" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="20">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:W100" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R77">
     <sortCondition ref="Q2"/>
   </sortState>

</xml_diff>

<commit_message>
added gaia robustness.. maybe
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{493AB0B3-DF4C-8643-BE7F-6065918041ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7148B1E-0D82-8844-854F-EB244557F6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2502,36 +2502,6 @@
       <c r="H32" t="s">
         <v>29</v>
       </c>
-      <c r="I32">
-        <v>5052</v>
-      </c>
-      <c r="J32">
-        <v>0.75</v>
-      </c>
-      <c r="K32">
-        <v>0.79</v>
-      </c>
-      <c r="L32">
-        <v>-0.02</v>
-      </c>
-      <c r="M32">
-        <v>4.49</v>
-      </c>
-      <c r="N32">
-        <v>300.1821223</v>
-      </c>
-      <c r="O32">
-        <v>22.7097759</v>
-      </c>
-      <c r="P32">
-        <v>19.7638</v>
-      </c>
-      <c r="Q32">
-        <v>7.67</v>
-      </c>
-      <c r="R32">
-        <v>7.41432</v>
-      </c>
       <c r="S32">
         <f t="shared" si="0"/>
         <v>349.61677638948368</v>

</xml_diff>

<commit_message>
finally finally gaia refactor. oida
</commit_message>
<xml_diff>
--- a/input/Targets_V10p1.xlsx
+++ b/input/Targets_V10p1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/WALTzER-simulator/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7148B1E-0D82-8844-854F-EB244557F6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23DF0F46-51BE-B44C-A6A1-AD3CA6FA5FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22840" yWindow="4740" windowWidth="33600" windowHeight="18900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="176">
   <si>
     <t>#pl_name</t>
   </si>
@@ -558,6 +558,12 @@
   </si>
   <si>
     <t>KELT-19 b</t>
+  </si>
+  <si>
+    <t>1242084170974175232 c</t>
+  </si>
+  <si>
+    <t>this is also WASP-14, but i dont want the name resolution</t>
   </si>
 </sst>
 </file>
@@ -963,7 +969,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BB110"/>
+  <dimension ref="A1:BB111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.83203125" bestFit="1" customWidth="1"/>
@@ -2502,12 +2508,42 @@
       <c r="H32" t="s">
         <v>29</v>
       </c>
+      <c r="I32">
+        <v>5052</v>
+      </c>
+      <c r="J32">
+        <v>0.75</v>
+      </c>
+      <c r="K32">
+        <v>0.79</v>
+      </c>
+      <c r="L32">
+        <v>-0.02</v>
+      </c>
+      <c r="M32">
+        <v>4.49</v>
+      </c>
+      <c r="N32">
+        <v>300.1821223</v>
+      </c>
+      <c r="O32">
+        <v>22.7097759</v>
+      </c>
+      <c r="P32">
+        <v>19.7638</v>
+      </c>
+      <c r="Q32">
+        <v>7.67</v>
+      </c>
+      <c r="R32">
+        <v>7.41432</v>
+      </c>
       <c r="S32">
-        <f t="shared" si="0"/>
+        <f>(0.000000000000000138*G32/(1.673534E-24*1.3*0.000000066726*F32*1.8986E+30/(E32*7149200000)^2))/100000</f>
         <v>349.61677638948368</v>
       </c>
       <c r="T32">
-        <f t="shared" si="1"/>
+        <f>IF(I32&gt;6800,-7,-5)</f>
         <v>-5</v>
       </c>
     </row>
@@ -5626,11 +5662,11 @@
         <v>9.6464700000000008</v>
       </c>
       <c r="S82">
-        <f t="shared" si="5"/>
+        <f>(0.000000000000000138*G82/(1.673534E-24*1.3*0.000000066726*F82*1.8986E+30/(E82*7149200000)^2))/100000</f>
         <v>103.20465157174387</v>
       </c>
       <c r="T82">
-        <f t="shared" si="4"/>
+        <f>IF(I82&gt;6800,-7,-5)</f>
         <v>-5</v>
       </c>
     </row>
@@ -6489,7 +6525,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>126</v>
       </c>
@@ -6553,7 +6589,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>131</v>
       </c>
@@ -6617,7 +6653,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>79</v>
       </c>
@@ -6681,7 +6717,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>107</v>
       </c>
@@ -6745,7 +6781,7 @@
         <v>-5</v>
       </c>
     </row>
-    <row r="101" spans="1:20" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:24" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>161</v>
       </c>
@@ -6765,7 +6801,7 @@
         <v>9.2583198549999999</v>
       </c>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>163</v>
       </c>
@@ -6797,7 +6833,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>164</v>
       </c>
@@ -6829,7 +6865,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>165</v>
       </c>
@@ -6861,7 +6897,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>166</v>
       </c>
@@ -6887,7 +6923,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>167</v>
       </c>
@@ -6913,7 +6949,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>168</v>
       </c>
@@ -6939,7 +6975,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>169</v>
       </c>
@@ -6965,7 +7001,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>170</v>
       </c>
@@ -6991,7 +7027,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>171</v>
       </c>
@@ -7015,6 +7051,20 @@
       </c>
       <c r="Q110">
         <v>19</v>
+      </c>
+    </row>
+    <row r="111" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="N111">
+        <v>218.27662916581701</v>
+      </c>
+      <c r="O111">
+        <v>21.8946865465029</v>
+      </c>
+      <c r="X111" s="1" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>